<commit_message>
Motore: requisiti datati e 'Una tra' (deroga Amato, Flessibile 0189/0195/0201/0202), esclusione domande solo operatori INPS, note requisiti
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZ53mE9kv9UaGeExs67Ewt
</commit_message>
<xml_diff>
--- a/motore/dati/Requisiti_domande_pensione.xlsx
+++ b/motore/dati/Requisiti_domande_pensione.xlsx
@@ -13548,7 +13548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13715,7 +13715,7 @@
       </c>
       <c r="L3" s="26" t="inlineStr">
         <is>
-          <t>Contributivo puro: 67 anni + 20 di contributi (importo ≥ 1,5 AS verificato in istruttoria) oppure 71 anni + 5 effettivi.</t>
+          <t>Requisiti da lista domande — età: 67; contributi: 20; inizio assicurazione: post 95; note: Esclusivamente contributivi (primo contributo dopo il 31/12/1995). A 67 anni: 20 anni di contributi e importo ≥ 1,5 volte l'assegno sociale; a 71 anni (con adeguamento dal 2027): 5 anni di contributi effettivi, senza soglia di importo.. Logica nel codice (predicato vecchiaiaContributiva).</t>
         </is>
       </c>
     </row>
@@ -13759,7 +13759,7 @@
       </c>
       <c r="L4" s="26" t="inlineStr">
         <is>
-          <t>Meno di 18 anni di contributi al 31/12/1995 + opzione certificata in FELPE; 67 anni + 20.</t>
+          <t>Requisiti da lista domande — età: 67; contributi: 20; soggettivo: Meno di 18 anni di contribuzione al 31/12/1995 ed esercizio dell'opzione per il calcolo contributivo (art. 1 c. 23 L. 335/1995); inizio assicurazione: ante 96; FELPE: si; note: Pensione interamente contributiva. Dal 2027 67 anni e 1 mese; dal 2028 67 anni e 3 mesi (adeguamento speranza di vita).. Logica nel codice (predicato opzioneContributivo).</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="L5" s="26" t="inlineStr">
         <is>
-          <t>Gestione separata + altre gestioni, meno di 18 anni al 1995, almeno 5 anni dopo il 1996: 67 anni + 15 (DM 282/1996 art. 3).</t>
+          <t>Requisiti da lista domande — età: 67; contributi: 20; soggettivo: meno di 18 anni di contribuzione al 31/12/1995 e almeno 15 anni di contributi di cui cinque dopo il 01/01/1996; inizio assicurazione: ante 96; note: Iscritto Gestione separata con periodi in altre gestioni. Logica nel codice (predicato computoGS).</t>
         </is>
       </c>
     </row>
@@ -13828,13 +13828,13 @@
       </c>
       <c r="E6" s="26" t="inlineStr">
         <is>
-          <t>ante96; deroghe</t>
+          <t>ante96</t>
         </is>
       </c>
       <c r="F6" s="26" t="inlineStr"/>
       <c r="G6" s="26" t="inlineStr">
         <is>
-          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età. | contr&gt;=15a =&gt; Servono 15 anni di contributi.</t>
+          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}). | contr&gt;=15a =&gt; Servono 15 anni di contributi (hai {x}). | una_tra(deroga.contr92 : 15 anni di contributi maturati entro il 31/12/1992 ; deroga.volontari92 : autorizzazione ai versamenti volontari entro il 31/12/1992 ; deroga.anz92 : 25 anni di anzianità assicurativa al 1992 con almeno 1 contributo prima del 1993) =&gt; Serve una tra le condizioni di deroga (deroghe Amato, art. 2 c. 3 D.Lgs. 503/1992):</t>
         </is>
       </c>
       <c r="H6" s="26" t="inlineStr">
@@ -13849,11 +13849,15 @@
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
-          <t>Deroga Amato dichiarata: bastano 15 anni di contributi.</t>
+          <t>Vecchiaia in deroga: età di vecchiaia, 15 anni di contributi e una delle condizioni Amato.</t>
         </is>
       </c>
       <c r="K6" s="26" t="inlineStr"/>
-      <c r="L6" s="26" t="inlineStr"/>
+      <c r="L6" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti dalla lista domande: età 67 (adeguata come la vecchiaia ordinaria), 15 anni di contributi, ante 96, e una tra le tre condizioni Amato (campo profilo "deroga": contr92, volontari92, anz92).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="26" t="inlineStr">
@@ -14131,7 +14135,7 @@
       </c>
       <c r="L12" s="26" t="inlineStr">
         <is>
-          <t>Contributivo puro: 64 anni + 20 di contributi (importo ≥ 3 AS verificato in istruttoria).</t>
+          <t>Requisiti da lista domande — età: 64; contributi: 20; soggettivo: Importo della prima rata non inferiore alla soglia prevista; inizio assicurazione: post 95; note: importo soglia. Logica nel codice (predicato anticipataContributiva).</t>
         </is>
       </c>
     </row>
@@ -14173,7 +14177,11 @@
           <t>anticipataComputoGS</t>
         </is>
       </c>
-      <c r="L13" s="26" t="inlineStr"/>
+      <c r="L13" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: 42 anni e 10 mesi fino al 2026; 42 anni e 11 mesi per il 2027; 43 anni e 1 mese per il 2028. (M) / 41 anni e 10 mesi fino al 2026; 41 anni e 11 mesi per il 2027; 42 anni e 1 mese per il 2028. (F); soggettivo: Iscritto alla Gestione separata con periodi in altre gestioni; meno di 18 anni di contribuzione al 31/12/1995; inizio assicurazione: ante 96; note: Computo in Gestione separata dei periodi in altre gestioni (art. 3 DM 282/1996); requisiti contributivi come anticipata ordinaria.. Logica nel codice (predicato anticipataComputoGS).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="26" t="inlineStr">
@@ -14213,7 +14221,11 @@
           <t>anticipataOpzioneContributivo</t>
         </is>
       </c>
-      <c r="L14" s="26" t="inlineStr"/>
+      <c r="L14" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — età: 64; contributi: 20; soggettivo: Meno di 18 anni di contribuzione al 31/12/1995 ed esercizio dell'opzione per il calcolo contributivo (art. 1 c. 23 L. 335/1995); inizio assicurazione: ante 96; FELPE: si; note: Pensione interamente contributiva: accesso a 64 anni con 20 di contributi e importo soglia (come 0017); in alternativa requisiti dell'anticipata ordinaria (42a10m uomini / 41a10m donne fino al 2026). Verificare condizioni dell'opzione.. Logica nel codice (predicato anticipataOpzioneContributivo).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="26" t="inlineStr">
@@ -14552,7 +14564,11 @@
       </c>
       <c r="E22" s="26" t="inlineStr"/>
       <c r="F22" s="26" t="inlineStr"/>
-      <c r="G22" s="26" t="inlineStr"/>
+      <c r="G22" s="26" t="inlineStr">
+        <is>
+          <t>eta@31/12/2025&gt;=62a =&gt; Servono 62 anni di età al 31/12/2025 (avevi {x}). | contr@31/12/2025&gt;=41a =&gt; Servono 41 anni di contributi al 31/12/2025 (avevi {x}).</t>
+        </is>
+      </c>
       <c r="H22" s="26" t="inlineStr">
         <is>
           <t>non_accessibile</t>
@@ -14563,27 +14579,27 @@
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J22" s="26" t="inlineStr"/>
-      <c r="K22" s="26" t="inlineStr">
-        <is>
-          <t>flessibile</t>
-        </is>
-      </c>
+      <c r="J22" s="26" t="inlineStr">
+        <is>
+          <t>Flessibile (Quota 103): 62 anni di età e 41 di contributi maturati entro il 31/12/2025 e requisiti raggiunti entro il 31/12/2025. Stima sui dati attuali: verificare in UNEX.</t>
+        </is>
+      </c>
+      <c r="K22" s="26" t="n"/>
       <c r="L22" s="26" t="inlineStr">
         <is>
-          <t>Quota 103: 62 anni + 41 di contributi maturati entro il 31/12/2025 (diritto acquisito, stima).</t>
+          <t>Lista domande: 62 anni e 41 di contributi al 31/12/2025; calcolo contributivo.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0190</t>
+          <t>0001-0001-0189</t>
         </is>
       </c>
       <c r="B23" s="26" t="inlineStr">
         <is>
-          <t>Pensione Anticipata opzione donna legge di bilancio 2023/2024/2025</t>
+          <t>Pensione Anticipata Flessibile</t>
         </is>
       </c>
       <c r="C23" s="26" t="inlineStr">
@@ -14594,9 +14610,13 @@
       <c r="D23" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E23" s="26" t="inlineStr"/>
-      <c r="F23" s="26" t="inlineStr"/>
-      <c r="G23" s="26" t="inlineStr"/>
+      <c r="E23" s="26" t="n"/>
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="26" t="inlineStr">
+        <is>
+          <t>eta@31/12/2023&gt;=62a =&gt; Servono 62 anni di età al 31/12/2023 (avevi {x}). | contr@31/12/2023&gt;=41a =&gt; Servono 41 anni di contributi al 31/12/2023 (avevi {x}).</t>
+        </is>
+      </c>
       <c r="H23" s="26" t="inlineStr">
         <is>
           <t>non_accessibile</t>
@@ -14607,27 +14627,27 @@
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J23" s="26" t="inlineStr"/>
-      <c r="K23" s="26" t="inlineStr">
-        <is>
-          <t>opzioneDonna</t>
-        </is>
-      </c>
+      <c r="J23" s="26" t="inlineStr">
+        <is>
+          <t>Flessibile (Quota 103): 62 anni di età e 41 di contributi maturati entro il 31/12/2023 e requisiti raggiunti entro il 31/12/2025. Stima sui dati attuali: verificare in UNEX.</t>
+        </is>
+      </c>
+      <c r="K23" s="26" t="n"/>
       <c r="L23" s="26" t="inlineStr">
         <is>
-          <t>Opzione donna: requisiti stimati al 31/12/2024 + condizione soggettiva; misura non rinnovata.</t>
+          <t>Lista domande: 62 anni e 41 di contributi al 31/12/2023; requisiti entro il 31/12/2025.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0162</t>
+          <t>0001-0001-0195</t>
         </is>
       </c>
       <c r="B24" s="26" t="inlineStr">
         <is>
-          <t>Pensione Anticipata Prepensionamento Editoria</t>
+          <t>Pensione Anticipata Flessibile opzione contributivo</t>
         </is>
       </c>
       <c r="C24" s="26" t="inlineStr">
@@ -14640,11 +14660,15 @@
       </c>
       <c r="E24" s="26" t="inlineStr">
         <is>
-          <t>editoria</t>
-        </is>
-      </c>
-      <c r="F24" s="26" t="inlineStr"/>
-      <c r="G24" s="26" t="inlineStr"/>
+          <t>ante96; cert.OPZIONE_CONTRIBUTIVO</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="n"/>
+      <c r="G24" s="26" t="inlineStr">
+        <is>
+          <t>eta@31/12/2025&gt;=62a =&gt; Servono 62 anni di età al 31/12/2025 (avevi {x}). | contr@31/12/2025&gt;=41a =&gt; Servono 41 anni di contributi al 31/12/2025 (avevi {x}).</t>
+        </is>
+      </c>
       <c r="H24" s="26" t="inlineStr">
         <is>
           <t>non_accessibile</t>
@@ -14652,26 +14676,30 @@
       </c>
       <c r="I24" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
+          <t>accessibile</t>
         </is>
       </c>
       <c r="J24" s="26" t="inlineStr">
         <is>
-          <t>Prepensionamento editoria dichiarato: verificare crisi aziendale accertata e CIGS per accordi di procedura.</t>
-        </is>
-      </c>
-      <c r="K24" s="26" t="inlineStr"/>
-      <c r="L24" s="26" t="inlineStr"/>
+          <t>Flessibile (Quota 103): 62 anni di età e 41 di contributi maturati entro il 31/12/2025 e requisiti raggiunti entro il 31/12/2025. Stima sui dati attuali: verificare in UNEX. Calcolo con opzione contributivo (FELPE).</t>
+        </is>
+      </c>
+      <c r="K24" s="26" t="n"/>
+      <c r="L24" s="26" t="inlineStr">
+        <is>
+          <t>Lista domande: 62+41 al 31/12/2025, ante 96, certificazione FELPE di opzione al contributivo (art. 1 c. 23 L. 335/1995).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0144</t>
+          <t>0001-0001-0202</t>
         </is>
       </c>
       <c r="B25" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità/anticipata con Salvaguardia ex L. 214</t>
+          <t>Pensione Anticipata Flessibile legge di bilancio 2024/2025 opzione contributivo</t>
         </is>
       </c>
       <c r="C25" s="26" t="inlineStr">
@@ -14684,18 +14712,18 @@
       </c>
       <c r="E25" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L214</t>
-        </is>
-      </c>
-      <c r="F25" s="26" t="inlineStr"/>
+          <t>ante96; cert.OPZIONE_CONTRIBUTIVO</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="n"/>
       <c r="G25" s="26" t="inlineStr">
         <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia L214 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
+          <t>eta@31/12/2025&gt;=62a =&gt; Servono 62 anni di età al 31/12/2025 (avevi {x}). | contr@31/12/2025&gt;=41a =&gt; Servono 41 anni di contributi al 31/12/2025 (avevi {x}).</t>
         </is>
       </c>
       <c r="H25" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
+          <t>non_accessibile</t>
         </is>
       </c>
       <c r="I25" s="26" t="inlineStr">
@@ -14705,21 +14733,25 @@
       </c>
       <c r="J25" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L214 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
-        </is>
-      </c>
-      <c r="K25" s="26" t="inlineStr"/>
-      <c r="L25" s="26" t="inlineStr"/>
+          <t>Flessibile (Quota 103): 62 anni di età e 41 di contributi maturati entro il 31/12/2025 e requisiti raggiunti entro il 31/12/2025. Stima sui dati attuali: verificare in UNEX. Calcolo con opzione contributivo (FELPE).</t>
+        </is>
+      </c>
+      <c r="K25" s="26" t="n"/>
+      <c r="L25" s="26" t="inlineStr">
+        <is>
+          <t>Lista domande: 62+41 al 31/12/2025, ante 96, certificazione FELPE di opzione al contributivo (art. 1 c. 23 L. 335/1995).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0145</t>
+          <t>0001-0001-0190</t>
         </is>
       </c>
       <c r="B26" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità/anticipata con Salvaguardia ex L. 135</t>
+          <t>Pensione Anticipata opzione donna legge di bilancio 2023/2024/2025</t>
         </is>
       </c>
       <c r="C26" s="26" t="inlineStr">
@@ -14730,20 +14762,12 @@
       <c r="D26" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E26" s="26" t="inlineStr">
-        <is>
-          <t>cert.SALVAGUARDIA; salv.L135</t>
-        </is>
-      </c>
+      <c r="E26" s="26" t="inlineStr"/>
       <c r="F26" s="26" t="inlineStr"/>
-      <c r="G26" s="26" t="inlineStr">
-        <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia L135 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
-        </is>
-      </c>
+      <c r="G26" s="26" t="inlineStr"/>
       <c r="H26" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
+          <t>non_accessibile</t>
         </is>
       </c>
       <c r="I26" s="26" t="inlineStr">
@@ -14751,23 +14775,27 @@
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J26" s="26" t="inlineStr">
-        <is>
-          <t>Salvaguardia L135 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
-        </is>
-      </c>
-      <c r="K26" s="26" t="inlineStr"/>
-      <c r="L26" s="26" t="inlineStr"/>
+      <c r="J26" s="26" t="inlineStr"/>
+      <c r="K26" s="26" t="inlineStr">
+        <is>
+          <t>opzioneDonna</t>
+        </is>
+      </c>
+      <c r="L26" s="26" t="inlineStr">
+        <is>
+          <t>Opzione donna: requisiti stimati al 31/12/2024 + condizione soggettiva; misura non rinnovata.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0146</t>
+          <t>0001-0001-0162</t>
         </is>
       </c>
       <c r="B27" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità/anticipata con Salvaguardia ex L. 228</t>
+          <t>Pensione Anticipata Prepensionamento Editoria</t>
         </is>
       </c>
       <c r="C27" s="26" t="inlineStr">
@@ -14780,28 +14808,24 @@
       </c>
       <c r="E27" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L228</t>
+          <t>editoria</t>
         </is>
       </c>
       <c r="F27" s="26" t="inlineStr"/>
-      <c r="G27" s="26" t="inlineStr">
-        <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia L228 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
-        </is>
-      </c>
+      <c r="G27" s="26" t="inlineStr"/>
       <c r="H27" s="26" t="inlineStr">
         <is>
+          <t>non_accessibile</t>
+        </is>
+      </c>
+      <c r="I27" s="26" t="inlineStr">
+        <is>
           <t>da_verificare</t>
         </is>
       </c>
-      <c r="I27" s="26" t="inlineStr">
-        <is>
-          <t>accessibile</t>
-        </is>
-      </c>
       <c r="J27" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L228 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
+          <t>Prepensionamento editoria dichiarato: verificare crisi aziendale accertata e CIGS per accordi di procedura.</t>
         </is>
       </c>
       <c r="K27" s="26" t="inlineStr"/>
@@ -14810,12 +14834,12 @@
     <row r="28">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0151</t>
+          <t>0001-0001-0144</t>
         </is>
       </c>
       <c r="B28" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità/anticipata con Salvaguardia D.L. 102/2013</t>
+          <t>Pensione di anzianità/anticipata con Salvaguardia ex L. 214</t>
         </is>
       </c>
       <c r="C28" s="26" t="inlineStr">
@@ -14828,13 +14852,13 @@
       </c>
       <c r="E28" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.DL102</t>
+          <t>cert.SALVAGUARDIA; salv.L214</t>
         </is>
       </c>
       <c r="F28" s="26" t="inlineStr"/>
       <c r="G28" s="26" t="inlineStr">
         <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia DL102 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia L214 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H28" s="26" t="inlineStr">
@@ -14849,7 +14873,7 @@
       </c>
       <c r="J28" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia DL102 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
+          <t>Salvaguardia L214 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K28" s="26" t="inlineStr"/>
@@ -14858,12 +14882,12 @@
     <row r="29">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0155</t>
+          <t>0001-0001-0145</t>
         </is>
       </c>
       <c r="B29" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità/anticipata con Salvaguardia legge 147/2013</t>
+          <t>Pensione di anzianità/anticipata con Salvaguardia ex L. 135</t>
         </is>
       </c>
       <c r="C29" s="26" t="inlineStr">
@@ -14876,13 +14900,13 @@
       </c>
       <c r="E29" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L147_2013</t>
+          <t>cert.SALVAGUARDIA; salv.L135</t>
         </is>
       </c>
       <c r="F29" s="26" t="inlineStr"/>
       <c r="G29" s="26" t="inlineStr">
         <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia L147_2013 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia L135 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H29" s="26" t="inlineStr">
@@ -14897,7 +14921,7 @@
       </c>
       <c r="J29" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L147_2013 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
+          <t>Salvaguardia L135 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K29" s="26" t="inlineStr"/>
@@ -14906,12 +14930,12 @@
     <row r="30">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0157</t>
+          <t>0001-0001-0146</t>
         </is>
       </c>
       <c r="B30" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità/anticipata con Salvaguardia legge 147/2014</t>
+          <t>Pensione di anzianità/anticipata con Salvaguardia ex L. 228</t>
         </is>
       </c>
       <c r="C30" s="26" t="inlineStr">
@@ -14924,13 +14948,13 @@
       </c>
       <c r="E30" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L147_2014</t>
+          <t>cert.SALVAGUARDIA; salv.L228</t>
         </is>
       </c>
       <c r="F30" s="26" t="inlineStr"/>
       <c r="G30" s="26" t="inlineStr">
         <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia L147_2014 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia L228 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H30" s="26" t="inlineStr">
@@ -14945,7 +14969,7 @@
       </c>
       <c r="J30" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L147_2014 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
+          <t>Salvaguardia L228 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K30" s="26" t="inlineStr"/>
@@ -14954,12 +14978,12 @@
     <row r="31">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0160</t>
+          <t>0001-0001-0151</t>
         </is>
       </c>
       <c r="B31" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità/anticipata con Salvaguardia   Legge 208/2015</t>
+          <t>Pensione di anzianità/anticipata con Salvaguardia D.L. 102/2013</t>
         </is>
       </c>
       <c r="C31" s="26" t="inlineStr">
@@ -14972,13 +14996,13 @@
       </c>
       <c r="E31" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L208</t>
+          <t>cert.SALVAGUARDIA; salv.DL102</t>
         </is>
       </c>
       <c r="F31" s="26" t="inlineStr"/>
       <c r="G31" s="26" t="inlineStr">
         <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia L208 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia DL102 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H31" s="26" t="inlineStr">
@@ -14993,7 +15017,7 @@
       </c>
       <c r="J31" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L208 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
+          <t>Salvaguardia DL102 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K31" s="26" t="inlineStr"/>
@@ -15002,12 +15026,12 @@
     <row r="32">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0165</t>
+          <t>0001-0001-0155</t>
         </is>
       </c>
       <c r="B32" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità/anticipata con Salvaguardia legge 232/2016</t>
+          <t>Pensione di anzianità/anticipata con Salvaguardia legge 147/2013</t>
         </is>
       </c>
       <c r="C32" s="26" t="inlineStr">
@@ -15020,13 +15044,13 @@
       </c>
       <c r="E32" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L232</t>
+          <t>cert.SALVAGUARDIA; salv.L147_2013</t>
         </is>
       </c>
       <c r="F32" s="26" t="inlineStr"/>
       <c r="G32" s="26" t="inlineStr">
         <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia L232 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia L147_2013 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H32" s="26" t="inlineStr">
@@ -15041,7 +15065,7 @@
       </c>
       <c r="J32" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L232 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
+          <t>Salvaguardia L147_2013 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K32" s="26" t="inlineStr"/>
@@ -15050,12 +15074,12 @@
     <row r="33">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>0001-0001-0181</t>
+          <t>0001-0001-0157</t>
         </is>
       </c>
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>Pensione di anzianità con Salvaguardia legge 178/2020</t>
+          <t>Pensione di anzianità/anticipata con Salvaguardia legge 147/2014</t>
         </is>
       </c>
       <c r="C33" s="26" t="inlineStr">
@@ -15068,13 +15092,13 @@
       </c>
       <c r="E33" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L178</t>
+          <t>cert.SALVAGUARDIA; salv.L147_2014</t>
         </is>
       </c>
       <c r="F33" s="26" t="inlineStr"/>
       <c r="G33" s="26" t="inlineStr">
         <is>
-          <t>contr&gt;=40a =&gt; Salvaguardia L178 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia L147_2014 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H33" s="26" t="inlineStr">
@@ -15089,7 +15113,7 @@
       </c>
       <c r="J33" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L178 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
+          <t>Salvaguardia L147_2014 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K33" s="26" t="inlineStr"/>
@@ -15098,12 +15122,12 @@
     <row r="34">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0144</t>
+          <t>0001-0001-0160</t>
         </is>
       </c>
       <c r="B34" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia con Salvaguardia ex L. 214</t>
+          <t>Pensione di anzianità/anticipata con Salvaguardia   Legge 208/2015</t>
         </is>
       </c>
       <c r="C34" s="26" t="inlineStr">
@@ -15116,18 +15140,18 @@
       </c>
       <c r="E34" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L214</t>
+          <t>cert.SALVAGUARDIA; salv.L208</t>
         </is>
       </c>
       <c r="F34" s="26" t="inlineStr"/>
       <c r="G34" s="26" t="inlineStr">
         <is>
-          <t>eta&gt;=M:65a/F:60a =&gt; Servono {min} di età (requisiti ante Fornero). | contr&gt;=20a =&gt; Servono 20 anni di contributi (15 con deroghe).</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia L208 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H34" s="26" t="inlineStr">
         <is>
-          <t>non_accessibile</t>
+          <t>da_verificare</t>
         </is>
       </c>
       <c r="I34" s="26" t="inlineStr">
@@ -15137,7 +15161,7 @@
       </c>
       <c r="J34" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L214 certificata in FELPE.</t>
+          <t>Salvaguardia L208 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K34" s="26" t="inlineStr"/>
@@ -15146,12 +15170,12 @@
     <row r="35">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0145</t>
+          <t>0001-0001-0165</t>
         </is>
       </c>
       <c r="B35" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia con Salvaguardia ex L. 135</t>
+          <t>Pensione di anzianità/anticipata con Salvaguardia legge 232/2016</t>
         </is>
       </c>
       <c r="C35" s="26" t="inlineStr">
@@ -15164,18 +15188,18 @@
       </c>
       <c r="E35" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L135</t>
+          <t>cert.SALVAGUARDIA; salv.L232</t>
         </is>
       </c>
       <c r="F35" s="26" t="inlineStr"/>
       <c r="G35" s="26" t="inlineStr">
         <is>
-          <t>eta&gt;=M:65a/F:60a =&gt; Servono {min} di età (requisiti ante Fornero). | contr&gt;=20a =&gt; Servono 20 anni di contributi (15 con deroghe).</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia L232 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H35" s="26" t="inlineStr">
         <is>
-          <t>non_accessibile</t>
+          <t>da_verificare</t>
         </is>
       </c>
       <c r="I35" s="26" t="inlineStr">
@@ -15185,7 +15209,7 @@
       </c>
       <c r="J35" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L135 certificata in FELPE.</t>
+          <t>Salvaguardia L232 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K35" s="26" t="inlineStr"/>
@@ -15194,12 +15218,12 @@
     <row r="36">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0146</t>
+          <t>0001-0001-0181</t>
         </is>
       </c>
       <c r="B36" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia con Salvaguardia ex L. 228</t>
+          <t>Pensione di anzianità con Salvaguardia legge 178/2020</t>
         </is>
       </c>
       <c r="C36" s="26" t="inlineStr">
@@ -15212,18 +15236,18 @@
       </c>
       <c r="E36" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L228</t>
+          <t>cert.SALVAGUARDIA; salv.L178</t>
         </is>
       </c>
       <c r="F36" s="26" t="inlineStr"/>
       <c r="G36" s="26" t="inlineStr">
         <is>
-          <t>eta&gt;=M:65a/F:60a =&gt; Servono {min} di età (requisiti ante Fornero). | contr&gt;=20a =&gt; Servono 20 anni di contributi (15 con deroghe).</t>
+          <t>contr&gt;=40a =&gt; Salvaguardia L178 certificata: servono 40 anni di contributi oppure quota 96/97 ({x} presenti). Verificare le quote.</t>
         </is>
       </c>
       <c r="H36" s="26" t="inlineStr">
         <is>
-          <t>non_accessibile</t>
+          <t>da_verificare</t>
         </is>
       </c>
       <c r="I36" s="26" t="inlineStr">
@@ -15233,7 +15257,7 @@
       </c>
       <c r="J36" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L228 certificata in FELPE.</t>
+          <t>Salvaguardia L178 certificata: 40 anni di contributi (requisiti ante Fornero).</t>
         </is>
       </c>
       <c r="K36" s="26" t="inlineStr"/>
@@ -15242,12 +15266,12 @@
     <row r="37">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0151</t>
+          <t>0001-0002-0144</t>
         </is>
       </c>
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia con Salvaguardia D.L. 102/2013</t>
+          <t>Pensione di vecchiaia con Salvaguardia ex L. 214</t>
         </is>
       </c>
       <c r="C37" s="26" t="inlineStr">
@@ -15260,7 +15284,7 @@
       </c>
       <c r="E37" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.DL102</t>
+          <t>cert.SALVAGUARDIA; salv.L214</t>
         </is>
       </c>
       <c r="F37" s="26" t="inlineStr"/>
@@ -15281,7 +15305,7 @@
       </c>
       <c r="J37" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia DL102 certificata in FELPE.</t>
+          <t>Salvaguardia L214 certificata in FELPE.</t>
         </is>
       </c>
       <c r="K37" s="26" t="inlineStr"/>
@@ -15290,12 +15314,12 @@
     <row r="38">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0155</t>
+          <t>0001-0002-0145</t>
         </is>
       </c>
       <c r="B38" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia  con Salvaguardia legge 147/2013</t>
+          <t>Pensione di vecchiaia con Salvaguardia ex L. 135</t>
         </is>
       </c>
       <c r="C38" s="26" t="inlineStr">
@@ -15308,7 +15332,7 @@
       </c>
       <c r="E38" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L147_2013</t>
+          <t>cert.SALVAGUARDIA; salv.L135</t>
         </is>
       </c>
       <c r="F38" s="26" t="inlineStr"/>
@@ -15329,7 +15353,7 @@
       </c>
       <c r="J38" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L147_2013 certificata in FELPE.</t>
+          <t>Salvaguardia L135 certificata in FELPE.</t>
         </is>
       </c>
       <c r="K38" s="26" t="inlineStr"/>
@@ -15338,12 +15362,12 @@
     <row r="39">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0157</t>
+          <t>0001-0002-0146</t>
         </is>
       </c>
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia  con Salvaguardia legge 147/2014</t>
+          <t>Pensione di vecchiaia con Salvaguardia ex L. 228</t>
         </is>
       </c>
       <c r="C39" s="26" t="inlineStr">
@@ -15356,7 +15380,7 @@
       </c>
       <c r="E39" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L147_2014</t>
+          <t>cert.SALVAGUARDIA; salv.L228</t>
         </is>
       </c>
       <c r="F39" s="26" t="inlineStr"/>
@@ -15377,7 +15401,7 @@
       </c>
       <c r="J39" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L147_2014 certificata in FELPE.</t>
+          <t>Salvaguardia L228 certificata in FELPE.</t>
         </is>
       </c>
       <c r="K39" s="26" t="inlineStr"/>
@@ -15386,12 +15410,12 @@
     <row r="40">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0165</t>
+          <t>0001-0002-0151</t>
         </is>
       </c>
       <c r="B40" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia con Salvaguardia legge 232/2016</t>
+          <t>Pensione di vecchiaia con Salvaguardia D.L. 102/2013</t>
         </is>
       </c>
       <c r="C40" s="26" t="inlineStr">
@@ -15404,7 +15428,7 @@
       </c>
       <c r="E40" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L232</t>
+          <t>cert.SALVAGUARDIA; salv.DL102</t>
         </is>
       </c>
       <c r="F40" s="26" t="inlineStr"/>
@@ -15425,7 +15449,7 @@
       </c>
       <c r="J40" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L232 certificata in FELPE.</t>
+          <t>Salvaguardia DL102 certificata in FELPE.</t>
         </is>
       </c>
       <c r="K40" s="26" t="inlineStr"/>
@@ -15434,12 +15458,12 @@
     <row r="41">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0181</t>
+          <t>0001-0002-0155</t>
         </is>
       </c>
       <c r="B41" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia con Salvaguardia legge 178/2020</t>
+          <t>Pensione di vecchiaia  con Salvaguardia legge 147/2013</t>
         </is>
       </c>
       <c r="C41" s="26" t="inlineStr">
@@ -15452,7 +15476,7 @@
       </c>
       <c r="E41" s="26" t="inlineStr">
         <is>
-          <t>cert.SALVAGUARDIA; salv.L178</t>
+          <t>cert.SALVAGUARDIA; salv.L147_2013</t>
         </is>
       </c>
       <c r="F41" s="26" t="inlineStr"/>
@@ -15473,7 +15497,7 @@
       </c>
       <c r="J41" s="26" t="inlineStr">
         <is>
-          <t>Salvaguardia L178 certificata in FELPE.</t>
+          <t>Salvaguardia L147_2013 certificata in FELPE.</t>
         </is>
       </c>
       <c r="K41" s="26" t="inlineStr"/>
@@ -15482,12 +15506,12 @@
     <row r="42">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0009</t>
+          <t>0001-0002-0157</t>
         </is>
       </c>
       <c r="B42" s="26" t="inlineStr">
         <is>
-          <t>Pensione supplementare di vecchiaia</t>
+          <t>Pensione di vecchiaia  con Salvaguardia legge 147/2014</t>
         </is>
       </c>
       <c r="C42" s="26" t="inlineStr">
@@ -15496,17 +15520,17 @@
         </is>
       </c>
       <c r="D42" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E42" s="26" t="inlineStr">
         <is>
-          <t>pensionato; noGest.GS</t>
+          <t>cert.SALVAGUARDIA; salv.L147_2014</t>
         </is>
       </c>
       <c r="F42" s="26" t="inlineStr"/>
       <c r="G42" s="26" t="inlineStr">
         <is>
-          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}).</t>
+          <t>eta&gt;=M:65a/F:60a =&gt; Servono {min} di età (requisiti ante Fornero). | contr&gt;=20a =&gt; Servono 20 anni di contributi (15 con deroghe).</t>
         </is>
       </c>
       <c r="H42" s="26" t="inlineStr">
@@ -15521,7 +15545,7 @@
       </c>
       <c r="J42" s="26" t="inlineStr">
         <is>
-          <t>Titolare di pensione diretta con contributi ulteriori: supplementare (domanda dopo 5 anni dalla decorrenza).</t>
+          <t>Salvaguardia L147_2014 certificata in FELPE.</t>
         </is>
       </c>
       <c r="K42" s="26" t="inlineStr"/>
@@ -15530,12 +15554,12 @@
     <row r="43">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0192</t>
+          <t>0001-0002-0165</t>
         </is>
       </c>
       <c r="B43" s="26" t="inlineStr">
         <is>
-          <t>Pensione supplementare di vecchiaia con computo Art. 3 D.M. 282/1996</t>
+          <t>Pensione di vecchiaia con Salvaguardia legge 232/2016</t>
         </is>
       </c>
       <c r="C43" s="26" t="inlineStr">
@@ -15544,17 +15568,17 @@
         </is>
       </c>
       <c r="D43" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E43" s="26" t="inlineStr">
         <is>
-          <t>pensionato; gest.GS</t>
+          <t>cert.SALVAGUARDIA; salv.L232</t>
         </is>
       </c>
       <c r="F43" s="26" t="inlineStr"/>
       <c r="G43" s="26" t="inlineStr">
         <is>
-          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}).</t>
+          <t>eta&gt;=M:65a/F:60a =&gt; Servono {min} di età (requisiti ante Fornero). | contr&gt;=20a =&gt; Servono 20 anni di contributi (15 con deroghe).</t>
         </is>
       </c>
       <c r="H43" s="26" t="inlineStr">
@@ -15569,7 +15593,7 @@
       </c>
       <c r="J43" s="26" t="inlineStr">
         <is>
-          <t>Supplementare con computo in Gestione separata (DM 282/1996).</t>
+          <t>Salvaguardia L232 certificata in FELPE.</t>
         </is>
       </c>
       <c r="K43" s="26" t="inlineStr"/>
@@ -15578,12 +15602,12 @@
     <row r="44">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0002</t>
+          <t>0001-0002-0181</t>
         </is>
       </c>
       <c r="B44" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia  a seguito di trasformazione A.O.I.</t>
+          <t>Pensione di vecchiaia con Salvaguardia legge 178/2020</t>
         </is>
       </c>
       <c r="C44" s="26" t="inlineStr">
@@ -15592,17 +15616,17 @@
         </is>
       </c>
       <c r="D44" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44" s="26" t="inlineStr">
         <is>
-          <t>titolareAOI</t>
+          <t>cert.SALVAGUARDIA; salv.L178</t>
         </is>
       </c>
       <c r="F44" s="26" t="inlineStr"/>
       <c r="G44" s="26" t="inlineStr">
         <is>
-          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}). | contr&gt;=20a =&gt; Servono 20 anni di contributi (hai {x}).</t>
+          <t>eta&gt;=M:65a/F:60a =&gt; Servono {min} di età (requisiti ante Fornero). | contr&gt;=20a =&gt; Servono 20 anni di contributi (15 con deroghe).</t>
         </is>
       </c>
       <c r="H44" s="26" t="inlineStr">
@@ -15617,7 +15641,7 @@
       </c>
       <c r="J44" s="26" t="inlineStr">
         <is>
-          <t>Trasformazione dell'assegno ordinario di invalidità in vecchiaia.</t>
+          <t>Salvaguardia L178 certificata in FELPE.</t>
         </is>
       </c>
       <c r="K44" s="26" t="inlineStr"/>
@@ -15626,12 +15650,12 @@
     <row r="45">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>0001-0002-0003</t>
+          <t>0001-0002-0009</t>
         </is>
       </c>
       <c r="B45" s="26" t="inlineStr">
         <is>
-          <t>Pensione di vecchiaia  a seguito di trasformazione Pensione di invalidità</t>
+          <t>Pensione supplementare di vecchiaia</t>
         </is>
       </c>
       <c r="C45" s="26" t="inlineStr">
@@ -15644,13 +15668,13 @@
       </c>
       <c r="E45" s="26" t="inlineStr">
         <is>
-          <t>titolareInvalidita</t>
+          <t>pensionato; noGest.GS</t>
         </is>
       </c>
       <c r="F45" s="26" t="inlineStr"/>
       <c r="G45" s="26" t="inlineStr">
         <is>
-          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}). | contr&gt;=20a =&gt; Servono 20 anni di contributi (hai {x}).</t>
+          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}).</t>
         </is>
       </c>
       <c r="H45" s="26" t="inlineStr">
@@ -15665,7 +15689,7 @@
       </c>
       <c r="J45" s="26" t="inlineStr">
         <is>
-          <t>Trasformazione della pensione di invalidità in vecchiaia.</t>
+          <t>Titolare di pensione diretta con contributi ulteriori: supplementare (domanda dopo 5 anni dalla decorrenza).</t>
         </is>
       </c>
       <c r="K45" s="26" t="inlineStr"/>
@@ -15674,29 +15698,33 @@
     <row r="46">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>0002-0011-0001</t>
+          <t>0001-0002-0192</t>
         </is>
       </c>
       <c r="B46" s="26" t="inlineStr">
         <is>
-          <t>Assegno ordinario di invalidità</t>
+          <t>Pensione supplementare di vecchiaia con computo Art. 3 D.M. 282/1996</t>
         </is>
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>invalidita</t>
+          <t>diretta</t>
         </is>
       </c>
       <c r="D46" s="26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E46" s="26" t="inlineStr">
         <is>
-          <t>grado.parziale</t>
+          <t>pensionato; gest.GS</t>
         </is>
       </c>
       <c r="F46" s="26" t="inlineStr"/>
-      <c r="G46" s="26" t="inlineStr"/>
+      <c r="G46" s="26" t="inlineStr">
+        <is>
+          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}).</t>
+        </is>
+      </c>
       <c r="H46" s="26" t="inlineStr">
         <is>
           <t>non_accessibile</t>
@@ -15707,44 +15735,44 @@
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J46" s="26" t="inlineStr"/>
-      <c r="K46" s="26" t="inlineStr">
-        <is>
-          <t>contributiInvalidita</t>
-        </is>
-      </c>
-      <c r="L46" s="26" t="inlineStr">
-        <is>
-          <t>Assegno ordinario: 5 anni di contributi, di cui 3 nell’ultimo quinquennio.</t>
-        </is>
-      </c>
+      <c r="J46" s="26" t="inlineStr">
+        <is>
+          <t>Supplementare con computo in Gestione separata (DM 282/1996).</t>
+        </is>
+      </c>
+      <c r="K46" s="26" t="inlineStr"/>
+      <c r="L46" s="26" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>0002-0011-0045</t>
+          <t>0001-0002-0002</t>
         </is>
       </c>
       <c r="B47" s="26" t="inlineStr">
         <is>
-          <t>Assegno ordinario di invalidità con computo Art. 3 D.M. 282/1996</t>
+          <t>Pensione di vecchiaia  a seguito di trasformazione A.O.I.</t>
         </is>
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>invalidita</t>
+          <t>diretta</t>
         </is>
       </c>
       <c r="D47" s="26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E47" s="26" t="inlineStr">
         <is>
-          <t>grado.parziale; gsPiuAltre</t>
+          <t>titolareAOI</t>
         </is>
       </c>
       <c r="F47" s="26" t="inlineStr"/>
-      <c r="G47" s="26" t="inlineStr"/>
+      <c r="G47" s="26" t="inlineStr">
+        <is>
+          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}). | contr&gt;=20a =&gt; Servono 20 anni di contributi (hai {x}).</t>
+        </is>
+      </c>
       <c r="H47" s="26" t="inlineStr">
         <is>
           <t>non_accessibile</t>
@@ -15755,44 +15783,44 @@
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J47" s="26" t="inlineStr"/>
-      <c r="K47" s="26" t="inlineStr">
-        <is>
-          <t>contributiInvalidita</t>
-        </is>
-      </c>
-      <c r="L47" s="26" t="inlineStr">
-        <is>
-          <t>Come sopra, con computo AGO + Gestione separata.</t>
-        </is>
-      </c>
+      <c r="J47" s="26" t="inlineStr">
+        <is>
+          <t>Trasformazione dell'assegno ordinario di invalidità in vecchiaia.</t>
+        </is>
+      </c>
+      <c r="K47" s="26" t="inlineStr"/>
+      <c r="L47" s="26" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>0002-0012-0001</t>
+          <t>0001-0002-0003</t>
         </is>
       </c>
       <c r="B48" s="26" t="inlineStr">
         <is>
-          <t>Pensione ordinaria di inabilità</t>
+          <t>Pensione di vecchiaia  a seguito di trasformazione Pensione di invalidità</t>
         </is>
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>invalidita</t>
+          <t>diretta</t>
         </is>
       </c>
       <c r="D48" s="26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E48" s="26" t="inlineStr">
         <is>
-          <t>grado.assoluta</t>
+          <t>titolareInvalidita</t>
         </is>
       </c>
       <c r="F48" s="26" t="inlineStr"/>
-      <c r="G48" s="26" t="inlineStr"/>
+      <c r="G48" s="26" t="inlineStr">
+        <is>
+          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}). | contr&gt;=20a =&gt; Servono 20 anni di contributi (hai {x}).</t>
+        </is>
+      </c>
       <c r="H48" s="26" t="inlineStr">
         <is>
           <t>non_accessibile</t>
@@ -15803,27 +15831,23 @@
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J48" s="26" t="inlineStr"/>
-      <c r="K48" s="26" t="inlineStr">
-        <is>
-          <t>contributiInvalidita</t>
-        </is>
-      </c>
-      <c r="L48" s="26" t="inlineStr">
-        <is>
-          <t>Pensione di inabilità: 5 anni di contributi, di cui 3 nell’ultimo quinquennio.</t>
-        </is>
-      </c>
+      <c r="J48" s="26" t="inlineStr">
+        <is>
+          <t>Trasformazione della pensione di invalidità in vecchiaia.</t>
+        </is>
+      </c>
+      <c r="K48" s="26" t="inlineStr"/>
+      <c r="L48" s="26" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>0002-0012-0045</t>
+          <t>0002-0011-0001</t>
         </is>
       </c>
       <c r="B49" s="26" t="inlineStr">
         <is>
-          <t>Pensione ordinaria di inabilità con computo Art. 3 D.M. 282/1996</t>
+          <t>Assegno ordinario di invalidità</t>
         </is>
       </c>
       <c r="C49" s="26" t="inlineStr">
@@ -15836,7 +15860,7 @@
       </c>
       <c r="E49" s="26" t="inlineStr">
         <is>
-          <t>grado.assoluta; gsPiuAltre</t>
+          <t>grado.parziale</t>
         </is>
       </c>
       <c r="F49" s="26" t="inlineStr"/>
@@ -15857,17 +15881,21 @@
           <t>contributiInvalidita</t>
         </is>
       </c>
-      <c r="L49" s="26" t="inlineStr"/>
+      <c r="L49" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: 5 di cui 3 nell'ultimo quinquennio; soggettivo: capacità lavorativa ridotta a meno di un terzo; note: Assegno di durata triennale, confermabile (dopo due conferme diviene definitivo); cumulabile con redditi da lavoro con riduzione. Art. 1 L. 222/1984.. Logica nel codice (predicato contributiInvalidita).</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>0002-0012-0052</t>
+          <t>0002-0011-0045</t>
         </is>
       </c>
       <c r="B50" s="26" t="inlineStr">
         <is>
-          <t>Pensione di Inabilità art. 2 comma 12 legge 335/1995</t>
+          <t>Assegno ordinario di invalidità con computo Art. 3 D.M. 282/1996</t>
         </is>
       </c>
       <c r="C50" s="26" t="inlineStr">
@@ -15880,7 +15908,7 @@
       </c>
       <c r="E50" s="26" t="inlineStr">
         <is>
-          <t>grado.assoluta; post95</t>
+          <t>grado.parziale; gsPiuAltre</t>
         </is>
       </c>
       <c r="F50" s="26" t="inlineStr"/>
@@ -15898,20 +15926,24 @@
       <c r="J50" s="26" t="inlineStr"/>
       <c r="K50" s="26" t="inlineStr">
         <is>
-          <t>inabilitaContributivoPuro</t>
-        </is>
-      </c>
-      <c r="L50" s="26" t="inlineStr"/>
+          <t>contributiInvalidita</t>
+        </is>
+      </c>
+      <c r="L50" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: 5 di cui 3 nell'ultimo quinquennio; soggettivo: capacità lavorativa ridotta a meno di un terzo; inizio assicurazione: ante 96; note: Iscritto Gestione separata con periodi in altre gestioni. Logica nel codice (predicato contributiInvalidita).</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>0002-0011-0005</t>
+          <t>0002-0012-0001</t>
         </is>
       </c>
       <c r="B51" s="26" t="inlineStr">
         <is>
-          <t>Assegno privilegiato di invalidità</t>
+          <t>Pensione ordinaria di inabilità</t>
         </is>
       </c>
       <c r="C51" s="26" t="inlineStr">
@@ -15920,11 +15952,11 @@
         </is>
       </c>
       <c r="D51" s="26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E51" s="26" t="inlineStr">
         <is>
-          <t>causaServizio; grado.parziale</t>
+          <t>grado.assoluta</t>
         </is>
       </c>
       <c r="F51" s="26" t="inlineStr"/>
@@ -15936,26 +15968,30 @@
       </c>
       <c r="I51" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
-        </is>
-      </c>
-      <c r="J51" s="26" t="inlineStr">
-        <is>
-          <t>Infermità dipendente da causa di servizio (gestione pubblica): assegno privilegiato, senza minimo contributivo.</t>
-        </is>
-      </c>
-      <c r="K51" s="26" t="inlineStr"/>
-      <c r="L51" s="26" t="inlineStr"/>
+          <t>accessibile</t>
+        </is>
+      </c>
+      <c r="J51" s="26" t="inlineStr"/>
+      <c r="K51" s="26" t="inlineStr">
+        <is>
+          <t>contributiInvalidita</t>
+        </is>
+      </c>
+      <c r="L51" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: 5 di cui 3 nell'ultimo quinquennio; soggettivo: assoluta e permanente impossibilità di svolgere qualsiasi attività lavorativa; note: Cessazione di ogni attività lavorativa; pensione ordinaria di inabilità (art. 2 L. 222/1984).. Logica nel codice (predicato contributiInvalidita).</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>0002-0012-0046</t>
+          <t>0002-0012-0045</t>
         </is>
       </c>
       <c r="B52" s="26" t="inlineStr">
         <is>
-          <t>Pensione di inabilità di privilegio Gestione Pubblica</t>
+          <t>Pensione ordinaria di inabilità con computo Art. 3 D.M. 282/1996</t>
         </is>
       </c>
       <c r="C52" s="26" t="inlineStr">
@@ -15964,11 +16000,11 @@
         </is>
       </c>
       <c r="D52" s="26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E52" s="26" t="inlineStr">
         <is>
-          <t>causaServizio; grado.assoluta; gest.ESCLUSIVA</t>
+          <t>grado.assoluta; gsPiuAltre</t>
         </is>
       </c>
       <c r="F52" s="26" t="inlineStr"/>
@@ -15980,26 +16016,30 @@
       </c>
       <c r="I52" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
-        </is>
-      </c>
-      <c r="J52" s="26" t="inlineStr">
-        <is>
-          <t>Inabilità per causa di servizio nella gestione pubblica (ex INPDAP).</t>
-        </is>
-      </c>
-      <c r="K52" s="26" t="inlineStr"/>
-      <c r="L52" s="26" t="inlineStr"/>
+          <t>accessibile</t>
+        </is>
+      </c>
+      <c r="J52" s="26" t="inlineStr"/>
+      <c r="K52" s="26" t="inlineStr">
+        <is>
+          <t>contributiInvalidita</t>
+        </is>
+      </c>
+      <c r="L52" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: 5 di cui 3 nell'ultimo quinquennio; soggettivo: assoluta e permanente impossibilità di svolgere qualsiasi attività lavorativa; inizio assicurazione: ante 96; note: Iscritto Gestione separata con periodi in altre gestioni. Logica nel codice (predicato contributiInvalidita).</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="26" t="inlineStr">
         <is>
-          <t>0002-0012-0005</t>
+          <t>0002-0012-0052</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
         <is>
-          <t>Pensione privilegiata di inabilità</t>
+          <t>Pensione di Inabilità art. 2 comma 12 legge 335/1995</t>
         </is>
       </c>
       <c r="C53" s="26" t="inlineStr">
@@ -16008,11 +16048,11 @@
         </is>
       </c>
       <c r="D53" s="26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E53" s="26" t="inlineStr">
         <is>
-          <t>causaServizio; grado.assoluta; noGest.ESCLUSIVA</t>
+          <t>grado.assoluta; post95</t>
         </is>
       </c>
       <c r="F53" s="26" t="inlineStr"/>
@@ -16024,26 +16064,30 @@
       </c>
       <c r="I53" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
-        </is>
-      </c>
-      <c r="J53" s="26" t="inlineStr">
-        <is>
-          <t>Pensione privilegiata di inabilità per causa di servizio.</t>
-        </is>
-      </c>
-      <c r="K53" s="26" t="inlineStr"/>
-      <c r="L53" s="26" t="inlineStr"/>
+          <t>accessibile</t>
+        </is>
+      </c>
+      <c r="J53" s="26" t="inlineStr"/>
+      <c r="K53" s="26" t="inlineStr">
+        <is>
+          <t>inabilitaContributivoPuro</t>
+        </is>
+      </c>
+      <c r="L53" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: 5 di cui 3 nell'ultimo quinquennio; soggettivo: Assoluta e permanente impossibilità di svolgere qualsiasi attività lavorativa; note: Art. 2 c. 12 L. 335/1995: pensione di inabilità con calcolo contributivo (maggiorazione fino ai 60 anni).. Logica nel codice (predicato inabilitaContributivoPuro).</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="26" t="inlineStr">
         <is>
-          <t>0002-0012-0047</t>
+          <t>0002-0011-0005</t>
         </is>
       </c>
       <c r="B54" s="26" t="inlineStr">
         <is>
-          <t>Pensione ordinaria di inabilità proficuo lavoro/mansioni gestione pubblica</t>
+          <t>Assegno privilegiato di invalidità</t>
         </is>
       </c>
       <c r="C54" s="26" t="inlineStr">
@@ -16056,7 +16100,7 @@
       </c>
       <c r="E54" s="26" t="inlineStr">
         <is>
-          <t>noCausaServizio; gest.ESCLUSIVA; grado.assoluta</t>
+          <t>causaServizio; grado.parziale</t>
         </is>
       </c>
       <c r="F54" s="26" t="inlineStr"/>
@@ -16073,7 +16117,7 @@
       </c>
       <c r="J54" s="26" t="inlineStr">
         <is>
-          <t>Gestione pubblica: inabilità a proficuo lavoro/mansioni per infermità non dipendente da causa di servizio. Verificare il minimo di servizio.</t>
+          <t>Infermità dipendente da causa di servizio (gestione pubblica): assegno privilegiato, senza minimo contributivo.</t>
         </is>
       </c>
       <c r="K54" s="26" t="inlineStr"/>
@@ -16082,12 +16126,12 @@
     <row r="55">
       <c r="A55" s="26" t="inlineStr">
         <is>
-          <t>0002-0012-0010</t>
+          <t>0002-0012-0046</t>
         </is>
       </c>
       <c r="B55" s="26" t="inlineStr">
         <is>
-          <t>Pensione di inabilità alla navigazione</t>
+          <t>Pensione di inabilità di privilegio Gestione Pubblica</t>
         </is>
       </c>
       <c r="C55" s="26" t="inlineStr">
@@ -16100,7 +16144,7 @@
       </c>
       <c r="E55" s="26" t="inlineStr">
         <is>
-          <t>marittimo; grado.assoluta</t>
+          <t>causaServizio; grado.assoluta; gest.ESCLUSIVA</t>
         </is>
       </c>
       <c r="F55" s="26" t="inlineStr"/>
@@ -16117,7 +16161,7 @@
       </c>
       <c r="J55" s="26" t="inlineStr">
         <is>
-          <t>Marittimo: inabilità alla navigazione, verificare la contribuzione marittima.</t>
+          <t>Inabilità per causa di servizio nella gestione pubblica (ex INPDAP).</t>
         </is>
       </c>
       <c r="K55" s="26" t="inlineStr"/>
@@ -16126,12 +16170,12 @@
     <row r="56">
       <c r="A56" s="26" t="inlineStr">
         <is>
-          <t>0002-0012-0168</t>
+          <t>0002-0012-0005</t>
         </is>
       </c>
       <c r="B56" s="26" t="inlineStr">
         <is>
-          <t>Pensione di Inabilità articolo 1 comma 250 legge 232/2016</t>
+          <t>Pensione privilegiata di inabilità</t>
         </is>
       </c>
       <c r="C56" s="26" t="inlineStr">
@@ -16144,7 +16188,7 @@
       </c>
       <c r="E56" s="26" t="inlineStr">
         <is>
-          <t>cert.AMIANTO; grado.assoluta</t>
+          <t>causaServizio; grado.assoluta; noGest.ESCLUSIVA</t>
         </is>
       </c>
       <c r="F56" s="26" t="inlineStr"/>
@@ -16161,7 +16205,7 @@
       </c>
       <c r="J56" s="26" t="inlineStr">
         <is>
-          <t>Esposizione all'amianto certificata: possibile pensione di inabilità ex art. 1 c. 250 L. 232/2016 (da verificare).</t>
+          <t>Pensione privilegiata di inabilità per causa di servizio.</t>
         </is>
       </c>
       <c r="K56" s="26" t="inlineStr"/>
@@ -16170,12 +16214,12 @@
     <row r="57">
       <c r="A57" s="26" t="inlineStr">
         <is>
-          <t>0002-0013-0009</t>
+          <t>0002-0012-0047</t>
         </is>
       </c>
       <c r="B57" s="26" t="inlineStr">
         <is>
-          <t>Pensione supplementare di invalidità</t>
+          <t>Pensione ordinaria di inabilità proficuo lavoro/mansioni gestione pubblica</t>
         </is>
       </c>
       <c r="C57" s="26" t="inlineStr">
@@ -16184,11 +16228,11 @@
         </is>
       </c>
       <c r="D57" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E57" s="26" t="inlineStr">
         <is>
-          <t>pensionato</t>
+          <t>noCausaServizio; gest.ESCLUSIVA; grado.assoluta</t>
         </is>
       </c>
       <c r="F57" s="26" t="inlineStr"/>
@@ -16205,7 +16249,7 @@
       </c>
       <c r="J57" s="26" t="inlineStr">
         <is>
-          <t>Già titolare di pensione: supplementare di invalidità sulla contribuzione ulteriore.</t>
+          <t>Gestione pubblica: inabilità a proficuo lavoro/mansioni per infermità non dipendente da causa di servizio. Verificare il minimo di servizio.</t>
         </is>
       </c>
       <c r="K57" s="26" t="inlineStr"/>
@@ -16214,12 +16258,12 @@
     <row r="58">
       <c r="A58" s="26" t="inlineStr">
         <is>
-          <t>0002-0013-0077</t>
+          <t>0002-0012-0010</t>
         </is>
       </c>
       <c r="B58" s="26" t="inlineStr">
         <is>
-          <t>Pensione di invalidità a carico di stato estero</t>
+          <t>Pensione di inabilità alla navigazione</t>
         </is>
       </c>
       <c r="C58" s="26" t="inlineStr">
@@ -16228,11 +16272,11 @@
         </is>
       </c>
       <c r="D58" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E58" s="26" t="inlineStr">
         <is>
-          <t>gest.ESTERO</t>
+          <t>marittimo; grado.assoluta</t>
         </is>
       </c>
       <c r="F58" s="26" t="inlineStr"/>
@@ -16249,7 +16293,7 @@
       </c>
       <c r="J58" s="26" t="inlineStr">
         <is>
-          <t>Periodi all'estero: prestazione a carico di Stato estero.</t>
+          <t>Marittimo: inabilità alla navigazione, verificare la contribuzione marittima.</t>
         </is>
       </c>
       <c r="K58" s="26" t="inlineStr"/>
@@ -16258,12 +16302,12 @@
     <row r="59">
       <c r="A59" s="26" t="inlineStr">
         <is>
-          <t>0002-0014-0001</t>
+          <t>0002-0012-0168</t>
         </is>
       </c>
       <c r="B59" s="26" t="inlineStr">
         <is>
-          <t>Riconoscimento di invalidità</t>
+          <t>Pensione di Inabilità articolo 1 comma 250 legge 232/2016</t>
         </is>
       </c>
       <c r="C59" s="26" t="inlineStr">
@@ -16272,11 +16316,11 @@
         </is>
       </c>
       <c r="D59" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E59" s="26" t="inlineStr">
         <is>
-          <t>soloRiconoscimento</t>
+          <t>cert.AMIANTO; grado.assoluta</t>
         </is>
       </c>
       <c r="F59" s="26" t="inlineStr"/>
@@ -16288,12 +16332,12 @@
       </c>
       <c r="I59" s="26" t="inlineStr">
         <is>
-          <t>accessibile</t>
+          <t>da_verificare</t>
         </is>
       </c>
       <c r="J59" s="26" t="inlineStr">
         <is>
-          <t>Domanda di solo riconoscimento dello stato di invalidità/inabilità, senza liquidazione di pensione.</t>
+          <t>Esposizione all'amianto certificata: possibile pensione di inabilità ex art. 1 c. 250 L. 232/2016 (da verificare).</t>
         </is>
       </c>
       <c r="K59" s="26" t="inlineStr"/>
@@ -16302,25 +16346,25 @@
     <row r="60">
       <c r="A60" s="26" t="inlineStr">
         <is>
-          <t>0003-0021-0001</t>
+          <t>0002-0013-0009</t>
         </is>
       </c>
       <c r="B60" s="26" t="inlineStr">
         <is>
-          <t>Pensione di reversibilità</t>
+          <t>Pensione supplementare di invalidità</t>
         </is>
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>superstiti</t>
+          <t>invalidita</t>
         </is>
       </c>
       <c r="D60" s="26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E60" s="26" t="inlineStr">
         <is>
-          <t>dante.pensionato</t>
+          <t>pensionato</t>
         </is>
       </c>
       <c r="F60" s="26" t="inlineStr"/>
@@ -16332,12 +16376,12 @@
       </c>
       <c r="I60" s="26" t="inlineStr">
         <is>
-          <t>accessibile</t>
+          <t>da_verificare</t>
         </is>
       </c>
       <c r="J60" s="26" t="inlineStr">
         <is>
-          <t>Il dante causa era titolare di pensione: reversibilità.</t>
+          <t>Già titolare di pensione: supplementare di invalidità sulla contribuzione ulteriore.</t>
         </is>
       </c>
       <c r="K60" s="26" t="inlineStr"/>
@@ -16346,17 +16390,17 @@
     <row r="61">
       <c r="A61" s="26" t="inlineStr">
         <is>
-          <t>0003-0021-0009</t>
+          <t>0002-0013-0077</t>
         </is>
       </c>
       <c r="B61" s="26" t="inlineStr">
         <is>
-          <t>Pensione supplementare di reversibilità</t>
+          <t>Pensione di invalidità a carico di stato estero</t>
         </is>
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>superstiti</t>
+          <t>invalidita</t>
         </is>
       </c>
       <c r="D61" s="26" t="n">
@@ -16364,7 +16408,7 @@
       </c>
       <c r="E61" s="26" t="inlineStr">
         <is>
-          <t>dante.pensionato; dante.supplementare</t>
+          <t>gest.ESTERO</t>
         </is>
       </c>
       <c r="F61" s="26" t="inlineStr"/>
@@ -16376,12 +16420,12 @@
       </c>
       <c r="I61" s="26" t="inlineStr">
         <is>
-          <t>accessibile</t>
+          <t>da_verificare</t>
         </is>
       </c>
       <c r="J61" s="26" t="inlineStr">
         <is>
-          <t>Il dante causa era titolare di pensione supplementare.</t>
+          <t>Periodi all'estero: prestazione a carico di Stato estero.</t>
         </is>
       </c>
       <c r="K61" s="26" t="inlineStr"/>
@@ -16390,25 +16434,25 @@
     <row r="62">
       <c r="A62" s="26" t="inlineStr">
         <is>
-          <t>0003-0022-0001</t>
+          <t>0002-0014-0001</t>
         </is>
       </c>
       <c r="B62" s="26" t="inlineStr">
         <is>
-          <t>Pensione indiretta</t>
+          <t>Riconoscimento di invalidità</t>
         </is>
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>superstiti</t>
+          <t>invalidita</t>
         </is>
       </c>
       <c r="D62" s="26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E62" s="26" t="inlineStr">
         <is>
-          <t>dante.noPensionato; noMarittimoScomparso</t>
+          <t>soloRiconoscimento</t>
         </is>
       </c>
       <c r="F62" s="26" t="inlineStr"/>
@@ -16423,27 +16467,23 @@
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J62" s="26" t="inlineStr"/>
-      <c r="K62" s="26" t="inlineStr">
-        <is>
-          <t>indiretta</t>
-        </is>
-      </c>
-      <c r="L62" s="26" t="inlineStr">
-        <is>
-          <t>Indiretta: 15 anni di contributi del dante causa, oppure 5 di cui 3 nell’ultimo quinquennio.</t>
-        </is>
-      </c>
+      <c r="J62" s="26" t="inlineStr">
+        <is>
+          <t>Domanda di solo riconoscimento dello stato di invalidità/inabilità, senza liquidazione di pensione.</t>
+        </is>
+      </c>
+      <c r="K62" s="26" t="inlineStr"/>
+      <c r="L62" s="26" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="26" t="inlineStr">
         <is>
-          <t>0003-0022-0045</t>
+          <t>0003-0021-0001</t>
         </is>
       </c>
       <c r="B63" s="26" t="inlineStr">
         <is>
-          <t>Pensione indiretta con computo Art. 3 D.M. 282/1996</t>
+          <t>Pensione di reversibilità</t>
         </is>
       </c>
       <c r="C63" s="26" t="inlineStr">
@@ -16456,7 +16496,7 @@
       </c>
       <c r="E63" s="26" t="inlineStr">
         <is>
-          <t>dante.noPensionato; dante.gsPiuAltre</t>
+          <t>dante.pensionato</t>
         </is>
       </c>
       <c r="F63" s="26" t="inlineStr"/>
@@ -16471,23 +16511,23 @@
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J63" s="26" t="inlineStr"/>
-      <c r="K63" s="26" t="inlineStr">
-        <is>
-          <t>indiretta</t>
-        </is>
-      </c>
+      <c r="J63" s="26" t="inlineStr">
+        <is>
+          <t>Il dante causa era titolare di pensione: reversibilità.</t>
+        </is>
+      </c>
+      <c r="K63" s="26" t="inlineStr"/>
       <c r="L63" s="26" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="26" t="inlineStr">
         <is>
-          <t>0003-0022-0005</t>
+          <t>0003-0021-0009</t>
         </is>
       </c>
       <c r="B64" s="26" t="inlineStr">
         <is>
-          <t>Pensione privilegiata indiretta</t>
+          <t>Pensione supplementare di reversibilità</t>
         </is>
       </c>
       <c r="C64" s="26" t="inlineStr">
@@ -16496,11 +16536,11 @@
         </is>
       </c>
       <c r="D64" s="26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E64" s="26" t="inlineStr">
         <is>
-          <t>dante.noPensionato; dante.causaServizio</t>
+          <t>dante.pensionato; dante.supplementare</t>
         </is>
       </c>
       <c r="F64" s="26" t="inlineStr"/>
@@ -16512,12 +16552,12 @@
       </c>
       <c r="I64" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
+          <t>accessibile</t>
         </is>
       </c>
       <c r="J64" s="26" t="inlineStr">
         <is>
-          <t>Decesso del dante causa per causa di servizio: pensione privilegiata indiretta.</t>
+          <t>Il dante causa era titolare di pensione supplementare.</t>
         </is>
       </c>
       <c r="K64" s="26" t="inlineStr"/>
@@ -16526,12 +16566,12 @@
     <row r="65">
       <c r="A65" s="26" t="inlineStr">
         <is>
-          <t>0003-0022-0046</t>
+          <t>0003-0022-0001</t>
         </is>
       </c>
       <c r="B65" s="26" t="inlineStr">
         <is>
-          <t>Pensione indiretta di privilegio Gestione Pubblica</t>
+          <t>Pensione indiretta</t>
         </is>
       </c>
       <c r="C65" s="26" t="inlineStr">
@@ -16540,11 +16580,11 @@
         </is>
       </c>
       <c r="D65" s="26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E65" s="26" t="inlineStr">
         <is>
-          <t>dante.noPensionato; dante.causaServizio; dante.esclusiva</t>
+          <t>dante.noPensionato; noMarittimoScomparso</t>
         </is>
       </c>
       <c r="F65" s="26" t="inlineStr"/>
@@ -16556,26 +16596,30 @@
       </c>
       <c r="I65" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
-        </is>
-      </c>
-      <c r="J65" s="26" t="inlineStr">
-        <is>
-          <t>Dante causa della gestione pubblica deceduto per causa di servizio.</t>
-        </is>
-      </c>
-      <c r="K65" s="26" t="inlineStr"/>
-      <c r="L65" s="26" t="inlineStr"/>
+          <t>accessibile</t>
+        </is>
+      </c>
+      <c r="J65" s="26" t="inlineStr"/>
+      <c r="K65" s="26" t="inlineStr">
+        <is>
+          <t>indiretta</t>
+        </is>
+      </c>
+      <c r="L65" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: 15 oppure 5 di cui 3 nell'ultimo quinquennio (del dante causa); soggettivo: Legame con il dante causa: coniuge (anche separato/divorziato con assegno e non risposato), figli minori/studenti/inabili, genitori ≥ 65 a carico, fratelli/sorelle inabili a carico. Logica nel codice (predicato indiretta).</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="26" t="inlineStr">
         <is>
-          <t>0003-0022-0052</t>
+          <t>0003-0022-0045</t>
         </is>
       </c>
       <c r="B66" s="26" t="inlineStr">
         <is>
-          <t>Pensione indiretta di inabilità ART.2, CO. 12, L. 335/95</t>
+          <t>Pensione indiretta con computo Art. 3 D.M. 282/1996</t>
         </is>
       </c>
       <c r="C66" s="26" t="inlineStr">
@@ -16584,11 +16628,11 @@
         </is>
       </c>
       <c r="D66" s="26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E66" s="26" t="inlineStr">
         <is>
-          <t>dante.noPensionato; dante.inabile</t>
+          <t>dante.noPensionato; dante.gsPiuAltre</t>
         </is>
       </c>
       <c r="F66" s="26" t="inlineStr"/>
@@ -16600,26 +16644,30 @@
       </c>
       <c r="I66" s="26" t="inlineStr">
         <is>
-          <t>da_verificare</t>
-        </is>
-      </c>
-      <c r="J66" s="26" t="inlineStr">
-        <is>
-          <t>Dante causa inabile al decesso (art. 2 c. 12 L. 335/1995): verificare i requisiti.</t>
-        </is>
-      </c>
-      <c r="K66" s="26" t="inlineStr"/>
-      <c r="L66" s="26" t="inlineStr"/>
+          <t>accessibile</t>
+        </is>
+      </c>
+      <c r="J66" s="26" t="inlineStr"/>
+      <c r="K66" s="26" t="inlineStr">
+        <is>
+          <t>indiretta</t>
+        </is>
+      </c>
+      <c r="L66" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: 15 oppure 5 di cui 3 nell'ultimo quinquennio (del dante causa); soggettivo: Legame con il dante causa: coniuge (anche separato/divorziato con assegno e non risposato), figli minori/studenti/inabili, genitori ≥ 65 a carico, fratelli/sorelle inabili a carico; dante causa iscritto alla Gestione separata con periodi in altre gestioni; inizio assicurazione: ante 96; note: Computo art. 3 DM 282/1996. Aliquota: 60% coniuge solo; 80% coniuge+1 figlio; 100% con 2 o più figli (o coniuge+2 figli) e simili. Riduzione per cumulo con redditi del beneficiario (25/40/50%, art. 1 c. 41 L. 335/1995).. Logica nel codice (predicato indiretta).</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="26" t="inlineStr">
         <is>
-          <t>0003-0023-0001</t>
+          <t>0003-0022-0005</t>
         </is>
       </c>
       <c r="B67" s="26" t="inlineStr">
         <is>
-          <t>Pensione ai superstiti di marittimo scomparso in mare</t>
+          <t>Pensione privilegiata indiretta</t>
         </is>
       </c>
       <c r="C67" s="26" t="inlineStr">
@@ -16632,7 +16680,7 @@
       </c>
       <c r="E67" s="26" t="inlineStr">
         <is>
-          <t>dante.marittimoScomparso</t>
+          <t>dante.noPensionato; dante.causaServizio</t>
         </is>
       </c>
       <c r="F67" s="26" t="inlineStr"/>
@@ -16644,12 +16692,12 @@
       </c>
       <c r="I67" s="26" t="inlineStr">
         <is>
-          <t>accessibile</t>
+          <t>da_verificare</t>
         </is>
       </c>
       <c r="J67" s="26" t="inlineStr">
         <is>
-          <t>Scomparsa in mare del marittimo, equiparata al decesso.</t>
+          <t>Decesso del dante causa per causa di servizio: pensione privilegiata indiretta.</t>
         </is>
       </c>
       <c r="K67" s="26" t="inlineStr"/>
@@ -16658,12 +16706,12 @@
     <row r="68">
       <c r="A68" s="26" t="inlineStr">
         <is>
-          <t>0003-0024-0077</t>
+          <t>0003-0022-0046</t>
         </is>
       </c>
       <c r="B68" s="26" t="inlineStr">
         <is>
-          <t>Pensione ai superstiti a carico di stato estero</t>
+          <t>Pensione indiretta di privilegio Gestione Pubblica</t>
         </is>
       </c>
       <c r="C68" s="26" t="inlineStr">
@@ -16672,11 +16720,11 @@
         </is>
       </c>
       <c r="D68" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E68" s="26" t="inlineStr">
         <is>
-          <t>dante.estero</t>
+          <t>dante.noPensionato; dante.causaServizio; dante.esclusiva</t>
         </is>
       </c>
       <c r="F68" s="26" t="inlineStr"/>
@@ -16693,7 +16741,7 @@
       </c>
       <c r="J68" s="26" t="inlineStr">
         <is>
-          <t>Pensione ai superstiti a carico di Stato estero.</t>
+          <t>Dante causa della gestione pubblica deceduto per causa di servizio.</t>
         </is>
       </c>
       <c r="K68" s="26" t="inlineStr"/>
@@ -16702,12 +16750,12 @@
     <row r="69">
       <c r="A69" s="26" t="inlineStr">
         <is>
-          <t>0003-0025-0001</t>
+          <t>0003-0022-0052</t>
         </is>
       </c>
       <c r="B69" s="26" t="inlineStr">
         <is>
-          <t>Indennità una tantum</t>
+          <t>Pensione indiretta di inabilità ART.2, CO. 12, L. 335/95</t>
         </is>
       </c>
       <c r="C69" s="26" t="inlineStr">
@@ -16716,11 +16764,11 @@
         </is>
       </c>
       <c r="D69" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E69" s="26" t="inlineStr">
         <is>
-          <t>dante.noPensionato; noMarittimoScomparso</t>
+          <t>dante.noPensionato; dante.inabile</t>
         </is>
       </c>
       <c r="F69" s="26" t="inlineStr"/>
@@ -16732,18 +16780,150 @@
       </c>
       <c r="I69" s="26" t="inlineStr">
         <is>
+          <t>da_verificare</t>
+        </is>
+      </c>
+      <c r="J69" s="26" t="inlineStr">
+        <is>
+          <t>Dante causa inabile al decesso (art. 2 c. 12 L. 335/1995): verificare i requisiti.</t>
+        </is>
+      </c>
+      <c r="K69" s="26" t="inlineStr"/>
+      <c r="L69" s="26" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="26" t="inlineStr">
+        <is>
+          <t>0003-0023-0001</t>
+        </is>
+      </c>
+      <c r="B70" s="26" t="inlineStr">
+        <is>
+          <t>Pensione ai superstiti di marittimo scomparso in mare</t>
+        </is>
+      </c>
+      <c r="C70" s="26" t="inlineStr">
+        <is>
+          <t>superstiti</t>
+        </is>
+      </c>
+      <c r="D70" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="E70" s="26" t="inlineStr">
+        <is>
+          <t>dante.marittimoScomparso</t>
+        </is>
+      </c>
+      <c r="F70" s="26" t="inlineStr"/>
+      <c r="G70" s="26" t="inlineStr"/>
+      <c r="H70" s="26" t="inlineStr">
+        <is>
+          <t>non_accessibile</t>
+        </is>
+      </c>
+      <c r="I70" s="26" t="inlineStr">
+        <is>
           <t>accessibile</t>
         </is>
       </c>
-      <c r="J69" s="26" t="inlineStr"/>
-      <c r="K69" s="26" t="inlineStr">
+      <c r="J70" s="26" t="inlineStr">
+        <is>
+          <t>Scomparsa in mare del marittimo, equiparata al decesso.</t>
+        </is>
+      </c>
+      <c r="K70" s="26" t="inlineStr"/>
+      <c r="L70" s="26" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="26" t="inlineStr">
+        <is>
+          <t>0003-0024-0077</t>
+        </is>
+      </c>
+      <c r="B71" s="26" t="inlineStr">
+        <is>
+          <t>Pensione ai superstiti a carico di stato estero</t>
+        </is>
+      </c>
+      <c r="C71" s="26" t="inlineStr">
+        <is>
+          <t>superstiti</t>
+        </is>
+      </c>
+      <c r="D71" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E71" s="26" t="inlineStr">
+        <is>
+          <t>dante.estero</t>
+        </is>
+      </c>
+      <c r="F71" s="26" t="inlineStr"/>
+      <c r="G71" s="26" t="inlineStr"/>
+      <c r="H71" s="26" t="inlineStr">
+        <is>
+          <t>non_accessibile</t>
+        </is>
+      </c>
+      <c r="I71" s="26" t="inlineStr">
+        <is>
+          <t>da_verificare</t>
+        </is>
+      </c>
+      <c r="J71" s="26" t="inlineStr">
+        <is>
+          <t>Pensione ai superstiti a carico di Stato estero.</t>
+        </is>
+      </c>
+      <c r="K71" s="26" t="inlineStr"/>
+      <c r="L71" s="26" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="26" t="inlineStr">
+        <is>
+          <t>0003-0025-0001</t>
+        </is>
+      </c>
+      <c r="B72" s="26" t="inlineStr">
+        <is>
+          <t>Indennità una tantum</t>
+        </is>
+      </c>
+      <c r="C72" s="26" t="inlineStr">
+        <is>
+          <t>superstiti</t>
+        </is>
+      </c>
+      <c r="D72" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E72" s="26" t="inlineStr">
+        <is>
+          <t>dante.noPensionato; noMarittimoScomparso</t>
+        </is>
+      </c>
+      <c r="F72" s="26" t="inlineStr"/>
+      <c r="G72" s="26" t="inlineStr"/>
+      <c r="H72" s="26" t="inlineStr">
+        <is>
+          <t>non_accessibile</t>
+        </is>
+      </c>
+      <c r="I72" s="26" t="inlineStr">
+        <is>
+          <t>accessibile</t>
+        </is>
+      </c>
+      <c r="J72" s="26" t="inlineStr"/>
+      <c r="K72" s="26" t="inlineStr">
         <is>
           <t>unaTantum</t>
         </is>
       </c>
-      <c r="L69" s="26" t="inlineStr">
-        <is>
-          <t>Indennità una tantum quando il dante causa non ha i requisiti per l’indiretta.</t>
+      <c r="L72" s="26" t="inlineStr">
+        <is>
+          <t>Requisiti da lista domande — contributi: n.d.; soggettivo: Superstiti dell'assicurato deceduto senza i requisiti per la pensione indiretta; note: Indennità una tantum. Logica nel codice (predicato unaTantum).</t>
         </is>
       </c>
     </row>
@@ -16789,7 +16969,7 @@
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>Requisiti: "tipo&gt;=soglia =&gt; messaggio" separati da " | ". Tipo: eta, contr (contributi), quota (età + contributi in anni). Soglia: 20a (anni), 6m (mesi), M:61a/F:56a (per sesso) oppure un parametro normativo (vecchiaia, contributiva64, anticipata, precoci, gravosiEta, usurantiEta) che il motore calcola per anno. Nel messaggio {min} = soglia, {x} = valore del richiedente.</t>
+          <t>Requisiti: "tipo&gt;=soglia =&gt; messaggio" separati da " | ". Tipo: eta, contr (contributi), quota (età + contributi in anni). Soglia: 20a (anni), 6m (mesi), M:61a/F:56a (per sesso) oppure un parametro normativo (vecchiaia, contributiva64, anticipata, precoci, gravosiEta, usurantiEta) che il motore calcola per anno. Nel messaggio {min} = soglia, {x} = valore del richiedente. Con data: "eta@31/12/2025&gt;=62a" / "contr@31/12/2025&gt;=41a" = requisito alla data indicata (stimato sui dati attuali). "Una tra": "una_tra(cond : testo ; cond : testo) =&gt; messaggio", vera se almeno una condizione è vera.</t>
         </is>
       </c>
     </row>
@@ -16824,7 +17004,7 @@
     <row r="9">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>Condizioni disponibili: ante96, post95, gest.X / noGest.X (AGO, GS, ESCLUSIVA, CASSA, ESTERO), gsPiuAltre, cert.X (PRECOCI, USURANTI, GRAVOSI, AMIANTO, SALVAGUARDIA, OPZIONE_CONTRIBUTIVO, VITTIMA_TERRORISMO), salv.CHIAVE, pensionato, titolareAOI, titolareInvalidita, deroghe, invalidita80, editoria, vittima80, noVittima80, sesso.F, grado.parziale/assoluta, causaServizio, noCausaServizio, marittimo, soloRiconoscimento, dante.pensionato/noPensionato/supplementare/causaServizio/marittimoScomparso/inabile/estero/esclusiva/gsPiuAltre, noMarittimoScomparso.</t>
+          <t>Condizioni disponibili: ante96, post95, gest.X / noGest.X (AGO, GS, ESCLUSIVA, CASSA, ESTERO), gsPiuAltre, cert.X (PRECOCI, USURANTI, GRAVOSI, AMIANTO, SALVAGUARDIA, OPZIONE_CONTRIBUTIVO, VITTIMA_TERRORISMO), salv.CHIAVE, pensionato, titolareAOI, titolareInvalidita, deroga.contr92 / deroga.volontari92 / deroga.anz92, invalidita80, editoria, vittima80, noVittima80, sesso.F, grado.parziale/assoluta, causaServizio, noCausaServizio, marittimo, soloRiconoscimento, dante.pensionato/noPensionato/supplementare/causaServizio/marittimoScomparso/inabile/estero/esclusiva/gsPiuAltre, noMarittimoScomparso.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deroga solo se manca la vecchiaia ordinaria; supplementari solo per titolari di pensione diretta (indicata nelle posizioni)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZ53mE9kv9UaGeExs67Ewt
</commit_message>
<xml_diff>
--- a/motore/dati/Requisiti_domande_pensione.xlsx
+++ b/motore/dati/Requisiti_domande_pensione.xlsx
@@ -13828,7 +13828,7 @@
       </c>
       <c r="E6" s="26" t="inlineStr">
         <is>
-          <t>ante96</t>
+          <t>ante96; noVecchiaiaOrdinaria; deroga.qualsiasi</t>
         </is>
       </c>
       <c r="F6" s="26" t="inlineStr"/>
@@ -13855,7 +13855,7 @@
       <c r="K6" s="26" t="inlineStr"/>
       <c r="L6" s="26" t="inlineStr">
         <is>
-          <t>Requisiti dalla lista domande: età 67 (adeguata come la vecchiaia ordinaria), 15 anni di contributi, ante 96, e una tra le tre condizioni Amato (campo profilo "deroga": contr92, volontari92, anz92).</t>
+          <t>Mostrata solo se: primo contributo ante 96, almeno una condizione Amato (15 anni di contributi entro il 31/12/1992, versamenti volontari autorizzati entro il 31/12/1992, 25 anni di anzianità assicurativa al 1992 con un contributo ante 1993) e NON si hanno già i requisiti della vecchiaia ordinaria (età + 20 anni). Requisiti: età di vecchiaia e 15 anni di contributi.</t>
         </is>
       </c>
     </row>
@@ -15693,7 +15693,11 @@
         </is>
       </c>
       <c r="K45" s="26" t="inlineStr"/>
-      <c r="L45" s="26" t="inlineStr"/>
+      <c r="L45" s="26" t="inlineStr">
+        <is>
+          <t>Solo per i titolari di pensione diretta (campo profilo "pensionato": vecchiaia/anzianità); non per AOI, invalidità o pensioni ai superstiti.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">
@@ -15741,7 +15745,11 @@
         </is>
       </c>
       <c r="K46" s="26" t="inlineStr"/>
-      <c r="L46" s="26" t="inlineStr"/>
+      <c r="L46" s="26" t="inlineStr">
+        <is>
+          <t>Solo per i titolari di pensione diretta (campo profilo "pensionato": vecchiaia/anzianità); non per AOI, invalidità o pensioni ai superstiti.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="26" t="inlineStr">
@@ -16385,7 +16393,11 @@
         </is>
       </c>
       <c r="K60" s="26" t="inlineStr"/>
-      <c r="L60" s="26" t="inlineStr"/>
+      <c r="L60" s="26" t="inlineStr">
+        <is>
+          <t>Solo per i titolari di pensione diretta.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="26" t="inlineStr">
@@ -17004,7 +17016,7 @@
     <row r="9">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>Condizioni disponibili: ante96, post95, gest.X / noGest.X (AGO, GS, ESCLUSIVA, CASSA, ESTERO), gsPiuAltre, cert.X (PRECOCI, USURANTI, GRAVOSI, AMIANTO, SALVAGUARDIA, OPZIONE_CONTRIBUTIVO, VITTIMA_TERRORISMO), salv.CHIAVE, pensionato, titolareAOI, titolareInvalidita, deroga.contr92 / deroga.volontari92 / deroga.anz92, invalidita80, editoria, vittima80, noVittima80, sesso.F, grado.parziale/assoluta, causaServizio, noCausaServizio, marittimo, soloRiconoscimento, dante.pensionato/noPensionato/supplementare/causaServizio/marittimoScomparso/inabile/estero/esclusiva/gsPiuAltre, noMarittimoScomparso.</t>
+          <t>Condizioni disponibili: ante96, post95, gest.X / noGest.X (AGO, GS, ESCLUSIVA, CASSA, ESTERO), gsPiuAltre, cert.X (PRECOCI, USURANTI, GRAVOSI, AMIANTO, SALVAGUARDIA, OPZIONE_CONTRIBUTIVO, VITTIMA_TERRORISMO), salv.CHIAVE, pensionato (titolare di pensione diretta), noVecchiaiaOrdinaria (non ha età+20 anni), deroga.qualsiasi, titolareAOI, titolareInvalidita, deroga.contr92 / deroga.volontari92 / deroga.anz92, invalidita80, editoria, vittima80, noVittima80, sesso.F, grado.parziale/assoluta, causaServizio, noCausaServizio, marittimo, soloRiconoscimento, dante.pensionato/noPensionato/supplementare/causaServizio/marittimoScomparso/inabile/estero/esclusiva/gsPiuAltre, noMarittimoScomparso.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: foglio 'Regole motore - variabili' con il significato di condizioni, requisiti e soglie
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZ53mE9kv9UaGeExs67Ewt
</commit_message>
<xml_diff>
--- a/motore/dati/Requisiti_domande_pensione.xlsx
+++ b/motore/dati/Requisiti_domande_pensione.xlsx
@@ -11,14 +11,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variabili e fonti" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regole motore" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regole motore - guida" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regole motore - variabili" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Variabili e fonti'!$A$4:$I$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Regole motore'!$A$1:$L$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Regole motore - variabili'!$A$1:$E$57</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="193" r:id="rId6"/>
+    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="193" r:id="rId7"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -26,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,6 +77,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -106,7 +112,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -129,11 +135,16 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="1" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -203,6 +214,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -16951,7 +16968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -17020,7 +17037,1575 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Il significato di ogni variabile (condizioni, tipi di requisito, soglie) è nel foglio "Regole motore - variabili".</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B1" s="25" t="inlineStr">
+        <is>
+          <t>Variabile</t>
+        </is>
+      </c>
+      <c r="C1" s="25" t="inlineStr">
+        <is>
+          <t>Significato</t>
+        </is>
+      </c>
+      <c r="D1" s="25" t="inlineStr">
+        <is>
+          <t>Da dove arriva il dato (campo del profilo)</t>
+        </is>
+      </c>
+      <c r="E1" s="25" t="inlineStr">
+        <is>
+          <t>Esempio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>ante96</t>
+        </is>
+      </c>
+      <c r="C2" s="27" t="inlineStr">
+        <is>
+          <t>Primo contributo entro il 31/12/1995: sistema di calcolo misto.</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>ante96 (dall'anno del primo contributo, archivio contributivo)</t>
+        </is>
+      </c>
+      <c r="E2" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: ante96</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>post95</t>
+        </is>
+      </c>
+      <c r="C3" s="27" t="inlineStr">
+        <is>
+          <t>Primo contributo dal 1996 in poi: sistema contributivo puro. È il contrario di ante96.</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="inlineStr">
+        <is>
+          <t>ante96 = falso</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>Esclusa se: post95 =&gt; Primo contributo dopo il 1995.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>sesso.F</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Il richiedente è donna (le soglie M/F si scelgono da sole con la sintassi M:…/F:…).</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>sesso</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: sesso.F</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>pensionato</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>È già titolare di una pensione DIRETTA (vecchiaia o anzianità). Non vale per AOI, invalidità o pensioni ai superstiti. Serve per le supplementari.</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>pensionato (derivato da pensioneDiretta nelle posizioni di prova)</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: pensionato</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>titolareAOI</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Titolare di assegno ordinario di invalidità (AOI): può chiedere la trasformazione in vecchiaia.</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>titolareAOI</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: titolareAOI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>titolareInvalidita</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>Titolare di pensione di invalidità del vecchio ordinamento: trasformazione in vecchiaia.</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>titolareInvalidita</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: titolareInvalidita</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>invalidita80</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>Invalidità riconosciuta pari o superiore all'80% (pensione anticipata di vecchiaia per invalidi).</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>invalidita80</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: invalidita80</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>editoria</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>Lavoratore del settore editoria con crisi aziendale: prepensionamento.</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>editoria</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: editoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>vittima80</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>Vittima del terrorismo con invalidità ≥ 80%.</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>vittimaInvalidita80 = vero</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: cert.VITTIMA_TERRORISMO; vittima80</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>noVittima80</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>Familiare di vittima del terrorismo o invalidità &lt; 80%. Contrario di vittima80.</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>vittimaInvalidita80 = falso</t>
+        </is>
+      </c>
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: cert.VITTIMA_TERRORISMO; noVittima80</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (richiedente)</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>noVecchiaiaOrdinaria</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>NON ha già i requisiti della vecchiaia ordinaria (età di vecchiaia e 20 anni di contributi). Serve a non mostrare la deroga a chi può chiedere la vecchiaia normale.</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>calcolata da età e contributi</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: ante96; noVecchiaiaOrdinaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (gestioni)</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>gest.AGO / noGest.AGO</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>Ha (o non ha) contributi nelle gestioni AGO: FPLD, artigiani, commercianti, agricoli.</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>gestioni (se vuoto si assume AGO)</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: gest.AGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (gestioni)</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>gest.GS / noGest.GS</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>Ha (o non ha) contributi nella Gestione separata.</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>gestioni</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: noGest.GS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (gestioni)</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>gest.ESCLUSIVA / noGest.ESCLUSIVA</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>Ha (o non ha) contributi in una forma esclusiva o esonerativa (ex INPDAP, ex ENPALS).</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>gestioni</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: gest.ESCLUSIVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (gestioni)</t>
+        </is>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>gest.CASSA / noGest.CASSA</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>Ha (o non ha) contributi in una cassa professionale privata.</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>gestioni</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: gest.CASSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (gestioni)</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>gest.ESTERO / noGest.ESTERO</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>Ha (o non ha) periodi di contribuzione all'estero.</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>gestioni</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: gest.ESTERO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (gestioni)</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>gsPiuAltre</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>Ha contributi in Gestione separata e in almeno un'altra gestione (AGO, esclusiva o cassa): serve il computo o la totalizzazione.</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>gestioni</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: gsPiuAltre</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (certificazioni FELPE)</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>cert.PRECOCI</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>Certificazione FELPE di lavoratore precoce.</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>felpe.certificazioni</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: cert.PRECOCI</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (certificazioni FELPE)</t>
+        </is>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>cert.USURANTI</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>Certificazione FELPE di lavori usuranti.</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>felpe.certificazioni</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: cert.USURANTI</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (certificazioni FELPE)</t>
+        </is>
+      </c>
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>cert.GRAVOSI</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>Certificazione FELPE di lavori gravosi.</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>felpe.certificazioni</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: cert.GRAVOSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (certificazioni FELPE)</t>
+        </is>
+      </c>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>cert.AMIANTO</t>
+        </is>
+      </c>
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>Certificazione FELPE di esposizione all'amianto.</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>felpe.certificazioni</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: cert.AMIANTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (certificazioni FELPE)</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="inlineStr">
+        <is>
+          <t>cert.OPZIONE_CONTRIBUTIVO</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>Certificazione FELPE dell'opzione per il calcolo contributivo (art. 1 c. 23 L. 335/1995).</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>felpe.certificazioni</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: ante96; cert.OPZIONE_CONTRIBUTIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (certificazioni FELPE)</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>cert.VITTIMA_TERRORISMO</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>Certificazione FELPE di vittima del terrorismo o delle stragi.</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>felpe.certificazioni</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: cert.VITTIMA_TERRORISMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (certificazioni FELPE)</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>cert.SALVAGUARDIA</t>
+        </is>
+      </c>
+      <c r="C25" s="27" t="inlineStr">
+        <is>
+          <t>Ha una certificazione FELPE di salvaguardia (qualunque legge).</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>felpe.certificazioni</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: cert.SALVAGUARDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (certificazioni FELPE)</t>
+        </is>
+      </c>
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>salv.CHIAVE</t>
+        </is>
+      </c>
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>Salvaguardia FELPE di una specifica legge. CHIAVE: L214, L135, L228, DL102, L147_2013, L147_2014, L208, L232, L178.</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>felpe.salvaguardia</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: salv.L214</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (deroghe Amato)</t>
+        </is>
+      </c>
+      <c r="B27" s="28" t="inlineStr">
+        <is>
+          <t>deroga.contr92</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="inlineStr">
+        <is>
+          <t>15 anni di contributi maturati entro il 31/12/1992.</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>deroga.contr92</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: deroga.contr92</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (deroghe Amato)</t>
+        </is>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>deroga.volontari92</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="inlineStr">
+        <is>
+          <t>Autorizzazione ai versamenti volontari entro il 31/12/1992.</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
+        <is>
+          <t>deroga.volontari92</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr">
+        <is>
+          <t>una_tra(deroga.volontari92 : … ; …)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (deroghe Amato)</t>
+        </is>
+      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>deroga.anz92</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="inlineStr">
+        <is>
+          <t>25 anni di anzianità assicurativa al 1992 con almeno un contributo prima del 1993.</t>
+        </is>
+      </c>
+      <c r="D29" s="27" t="inlineStr">
+        <is>
+          <t>deroga.anz92</t>
+        </is>
+      </c>
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>una_tra(deroga.anz92 : … ; …)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (deroghe Amato)</t>
+        </is>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>deroga.qualsiasi</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="inlineStr">
+        <is>
+          <t>Almeno una delle tre condizioni Amato è vera.</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>deroga.*</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: deroga.qualsiasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (invalidità)</t>
+        </is>
+      </c>
+      <c r="B31" s="28" t="inlineStr">
+        <is>
+          <t>grado.parziale / grado.assoluta</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>Grado di riduzione della capacità lavorativa: parziale (meno di un terzo: assegno) o assoluta e permanente (inabilità).</t>
+        </is>
+      </c>
+      <c r="D31" s="27" t="inlineStr">
+        <is>
+          <t>invalidita.grado</t>
+        </is>
+      </c>
+      <c r="E31" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: grado.assoluta</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (invalidità)</t>
+        </is>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>causaServizio / noCausaServizio</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>L'invalidità dipende (o non dipende) da causa di servizio.</t>
+        </is>
+      </c>
+      <c r="D32" s="27" t="inlineStr">
+        <is>
+          <t>invalidita.causaServizio</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="inlineStr">
+        <is>
+          <t>Esclusa se: causaServizio =&gt; …</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (invalidità)</t>
+        </is>
+      </c>
+      <c r="B33" s="28" t="inlineStr">
+        <is>
+          <t>marittimo</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>Il richiedente è un marittimo.</t>
+        </is>
+      </c>
+      <c r="D33" s="27" t="inlineStr">
+        <is>
+          <t>invalidita.marittimo</t>
+        </is>
+      </c>
+      <c r="E33" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: marittimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (invalidità)</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>soloRiconoscimento</t>
+        </is>
+      </c>
+      <c r="C34" s="27" t="inlineStr">
+        <is>
+          <t>Chiede solo il riconoscimento dello stato di invalidità, senza liquidazione di pensione.</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>invalidita.soloRiconoscimento</t>
+        </is>
+      </c>
+      <c r="E34" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: soloRiconoscimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (superstiti: persona deceduta)</t>
+        </is>
+      </c>
+      <c r="B35" s="28" t="inlineStr">
+        <is>
+          <t>dante.pensionato / dante.noPensionato</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>La persona deceduta (dante causa) era (o non era) titolare di pensione: reversibilità se era pensionato, indiretta se era un lavoratore.</t>
+        </is>
+      </c>
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>superstiti.dante.pensionato</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: dante.noPensionato</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (superstiti: persona deceduta)</t>
+        </is>
+      </c>
+      <c r="B36" s="28" t="inlineStr">
+        <is>
+          <t>dante.supplementare</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="inlineStr">
+        <is>
+          <t>Il dante causa era titolare di pensione supplementare.</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>superstiti.dante.titolareSupplementare</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: dante.pensionato; dante.supplementare</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (superstiti: persona deceduta)</t>
+        </is>
+      </c>
+      <c r="B37" s="28" t="inlineStr">
+        <is>
+          <t>dante.causaServizio</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>Il decesso o l'invalidità del dante causa dipendono da causa di servizio.</t>
+        </is>
+      </c>
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>superstiti.dante.causaServizio</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: dante.causaServizio</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (superstiti: persona deceduta)</t>
+        </is>
+      </c>
+      <c r="B38" s="28" t="inlineStr">
+        <is>
+          <t>dante.marittimoScomparso / noMarittimoScomparso</t>
+        </is>
+      </c>
+      <c r="C38" s="27" t="inlineStr">
+        <is>
+          <t>Il dante causa è un marittimo scomparso (o non lo è).</t>
+        </is>
+      </c>
+      <c r="D38" s="27" t="inlineStr">
+        <is>
+          <t>superstiti.dante.marittimoScomparso</t>
+        </is>
+      </c>
+      <c r="E38" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: noMarittimoScomparso</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (superstiti: persona deceduta)</t>
+        </is>
+      </c>
+      <c r="B39" s="28" t="inlineStr">
+        <is>
+          <t>dante.inabile</t>
+        </is>
+      </c>
+      <c r="C39" s="27" t="inlineStr">
+        <is>
+          <t>Il dante causa era inabile al momento del decesso.</t>
+        </is>
+      </c>
+      <c r="D39" s="27" t="inlineStr">
+        <is>
+          <t>superstiti.dante.inabileAlDecesso</t>
+        </is>
+      </c>
+      <c r="E39" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: dante.inabile</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (superstiti: persona deceduta)</t>
+        </is>
+      </c>
+      <c r="B40" s="28" t="inlineStr">
+        <is>
+          <t>dante.estero</t>
+        </is>
+      </c>
+      <c r="C40" s="27" t="inlineStr">
+        <is>
+          <t>Il dante causa aveva periodi di contribuzione all'estero.</t>
+        </is>
+      </c>
+      <c r="D40" s="27" t="inlineStr">
+        <is>
+          <t>superstiti.dante.gestioni contiene ESTERO</t>
+        </is>
+      </c>
+      <c r="E40" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: dante.estero</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (superstiti: persona deceduta)</t>
+        </is>
+      </c>
+      <c r="B41" s="28" t="inlineStr">
+        <is>
+          <t>dante.esclusiva</t>
+        </is>
+      </c>
+      <c r="C41" s="27" t="inlineStr">
+        <is>
+          <t>Il dante causa aveva contributi in forma esclusiva.</t>
+        </is>
+      </c>
+      <c r="D41" s="27" t="inlineStr">
+        <is>
+          <t>superstiti.dante.gestioni contiene ESCLUSIVA</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: dante.esclusiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="27" t="inlineStr">
+        <is>
+          <t>Condizione (superstiti: persona deceduta)</t>
+        </is>
+      </c>
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>dante.gsPiuAltre</t>
+        </is>
+      </c>
+      <c r="C42" s="27" t="inlineStr">
+        <is>
+          <t>Il dante causa aveva Gestione separata più un'altra gestione.</t>
+        </is>
+      </c>
+      <c r="D42" s="27" t="inlineStr">
+        <is>
+          <t>superstiti.dante.gestioni</t>
+        </is>
+      </c>
+      <c r="E42" s="27" t="inlineStr">
+        <is>
+          <t>Si applica se: dante.gsPiuAltre</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>Tipo di requisito</t>
+        </is>
+      </c>
+      <c r="B43" s="28" t="inlineStr">
+        <is>
+          <t>eta</t>
+        </is>
+      </c>
+      <c r="C43" s="27" t="inlineStr">
+        <is>
+          <t>Età del richiedente.</t>
+        </is>
+      </c>
+      <c r="D43" s="27" t="inlineStr">
+        <is>
+          <t>dataNascita</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr">
+        <is>
+          <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="27" t="inlineStr">
+        <is>
+          <t>Tipo di requisito</t>
+        </is>
+      </c>
+      <c r="B44" s="28" t="inlineStr">
+        <is>
+          <t>contr</t>
+        </is>
+      </c>
+      <c r="C44" s="27" t="inlineStr">
+        <is>
+          <t>Anzianità contributiva totale del richiedente.</t>
+        </is>
+      </c>
+      <c r="D44" s="27" t="inlineStr">
+        <is>
+          <t>contributi (anni, mesi)</t>
+        </is>
+      </c>
+      <c r="E44" s="27" t="inlineStr">
+        <is>
+          <t>contr&gt;=20a =&gt; Servono 20 anni di contributi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="inlineStr">
+        <is>
+          <t>Tipo di requisito</t>
+        </is>
+      </c>
+      <c r="B45" s="28" t="inlineStr">
+        <is>
+          <t>quota</t>
+        </is>
+      </c>
+      <c r="C45" s="27" t="inlineStr">
+        <is>
+          <t>Somma di età e contributi, in anni.</t>
+        </is>
+      </c>
+      <c r="D45" s="27" t="inlineStr">
+        <is>
+          <t>calcolata</t>
+        </is>
+      </c>
+      <c r="E45" s="27" t="inlineStr">
+        <is>
+          <t>quota&gt;=97.6 =&gt; Quota {min} (hai {x}).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>Tipo di requisito</t>
+        </is>
+      </c>
+      <c r="B46" s="28" t="inlineStr">
+        <is>
+          <t>@data (es. eta@31/12/2025&gt;=62a)</t>
+        </is>
+      </c>
+      <c r="C46" s="27" t="inlineStr">
+        <is>
+          <t>Requisito misurato a una data passata (stimato assumendo contribuzione continua). Se manca non maturerà più.</t>
+        </is>
+      </c>
+      <c r="D46" s="27" t="inlineStr">
+        <is>
+          <t>calcolata</t>
+        </is>
+      </c>
+      <c r="E46" s="27" t="inlineStr">
+        <is>
+          <t>contr@31/12/2025&gt;=41a =&gt; …</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>Tipo di requisito</t>
+        </is>
+      </c>
+      <c r="B47" s="28" t="inlineStr">
+        <is>
+          <t>una_tra(cond : testo ; …)</t>
+        </is>
+      </c>
+      <c r="C47" s="27" t="inlineStr">
+        <is>
+          <t>Il requisito è soddisfatto se almeno una delle condizioni elencate è vera.</t>
+        </is>
+      </c>
+      <c r="D47" s="27" t="inlineStr">
+        <is>
+          <t>condizioni sopra</t>
+        </is>
+      </c>
+      <c r="E47" s="27" t="inlineStr">
+        <is>
+          <t>una_tra(deroga.contr92 : 15 anni al 1992 ; deroga.anz92 : 25 anni di anzianità) =&gt; Serve una tra…</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>Soglia</t>
+        </is>
+      </c>
+      <c r="B48" s="28" t="inlineStr">
+        <is>
+          <t>20a, 6m</t>
+        </is>
+      </c>
+      <c r="C48" s="27" t="inlineStr">
+        <is>
+          <t>Soglia fissa in anni (a) o in mesi (m).</t>
+        </is>
+      </c>
+      <c r="D48" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="27" t="inlineStr">
+        <is>
+          <t>contr&gt;=20a</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>Soglia</t>
+        </is>
+      </c>
+      <c r="B49" s="28" t="inlineStr">
+        <is>
+          <t>M:61a/F:56a</t>
+        </is>
+      </c>
+      <c r="C49" s="27" t="inlineStr">
+        <is>
+          <t>Soglia diversa per uomini (M) e donne (F).</t>
+        </is>
+      </c>
+      <c r="D49" s="27" t="inlineStr">
+        <is>
+          <t>sesso</t>
+        </is>
+      </c>
+      <c r="E49" s="27" t="inlineStr">
+        <is>
+          <t>eta&gt;=M:61a/F:56a</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>Soglia</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="inlineStr">
+        <is>
+          <t>97.6</t>
+        </is>
+      </c>
+      <c r="C50" s="27" t="inlineStr">
+        <is>
+          <t>Numero puro: usato per la quota.</t>
+        </is>
+      </c>
+      <c r="D50" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="27" t="inlineStr">
+        <is>
+          <t>quota&gt;=97.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>Soglia (parametro normativo)</t>
+        </is>
+      </c>
+      <c r="B51" s="28" t="inlineStr">
+        <is>
+          <t>vecchiaia</t>
+        </is>
+      </c>
+      <c r="C51" s="27" t="inlineStr">
+        <is>
+          <t>67 anni più l'adeguamento alla speranza di vita (+1 mese dal 2027, +3 dal 2028).</t>
+        </is>
+      </c>
+      <c r="D51" s="27" t="inlineStr">
+        <is>
+          <t>calcolato per anno</t>
+        </is>
+      </c>
+      <c r="E51" s="27" t="inlineStr">
+        <is>
+          <t>eta&gt;=vecchiaia</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t>Soglia (parametro normativo)</t>
+        </is>
+      </c>
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>vecchiaiaContributiva71</t>
+        </is>
+      </c>
+      <c r="C52" s="27" t="inlineStr">
+        <is>
+          <t>71 anni più adeguamento: vecchiaia contributiva con importo ridotto.</t>
+        </is>
+      </c>
+      <c r="D52" s="27" t="inlineStr">
+        <is>
+          <t>calcolato per anno</t>
+        </is>
+      </c>
+      <c r="E52" s="27" t="inlineStr">
+        <is>
+          <t>eta&gt;=vecchiaiaContributiva71</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>Soglia (parametro normativo)</t>
+        </is>
+      </c>
+      <c r="B53" s="28" t="inlineStr">
+        <is>
+          <t>contributiva64</t>
+        </is>
+      </c>
+      <c r="C53" s="27" t="inlineStr">
+        <is>
+          <t>64 anni più adeguamento: anticipata nel sistema contributivo puro (con 20 anni).</t>
+        </is>
+      </c>
+      <c r="D53" s="27" t="inlineStr">
+        <is>
+          <t>calcolato per anno</t>
+        </is>
+      </c>
+      <c r="E53" s="27" t="inlineStr">
+        <is>
+          <t>eta&gt;=contributiva64</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="27" t="inlineStr">
+        <is>
+          <t>Soglia (parametro normativo)</t>
+        </is>
+      </c>
+      <c r="B54" s="28" t="inlineStr">
+        <is>
+          <t>anticipata</t>
+        </is>
+      </c>
+      <c r="C54" s="27" t="inlineStr">
+        <is>
+          <t>Contributi per l'anticipata ordinaria: 42 anni e 10 mesi (uomini), 41 anni e 10 mesi (donne), più adeguamento.</t>
+        </is>
+      </c>
+      <c r="D54" s="27" t="inlineStr">
+        <is>
+          <t>calcolato per anno e sesso</t>
+        </is>
+      </c>
+      <c r="E54" s="27" t="inlineStr">
+        <is>
+          <t>contr&gt;=anticipata</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="27" t="inlineStr">
+        <is>
+          <t>Soglia (parametro normativo)</t>
+        </is>
+      </c>
+      <c r="B55" s="28" t="inlineStr">
+        <is>
+          <t>precoci</t>
+        </is>
+      </c>
+      <c r="C55" s="27" t="inlineStr">
+        <is>
+          <t>41 anni di contributi più adeguamento (lavoratori precoci).</t>
+        </is>
+      </c>
+      <c r="D55" s="27" t="inlineStr">
+        <is>
+          <t>calcolato per anno</t>
+        </is>
+      </c>
+      <c r="E55" s="27" t="inlineStr">
+        <is>
+          <t>contr&gt;=precoci</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="27" t="inlineStr">
+        <is>
+          <t>Soglia (parametro normativo)</t>
+        </is>
+      </c>
+      <c r="B56" s="28" t="inlineStr">
+        <is>
+          <t>gravosiEta</t>
+        </is>
+      </c>
+      <c r="C56" s="27" t="inlineStr">
+        <is>
+          <t>66 anni e 7 mesi: età per i lavori gravosi (non adeguata).</t>
+        </is>
+      </c>
+      <c r="D56" s="27" t="inlineStr">
+        <is>
+          <t>fisso</t>
+        </is>
+      </c>
+      <c r="E56" s="27" t="inlineStr">
+        <is>
+          <t>eta&gt;=gravosiEta</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="27" t="inlineStr">
+        <is>
+          <t>Soglia (parametro normativo)</t>
+        </is>
+      </c>
+      <c r="B57" s="28" t="inlineStr">
+        <is>
+          <t>usurantiEta</t>
+        </is>
+      </c>
+      <c r="C57" s="27" t="inlineStr">
+        <is>
+          <t>61 anni e 7 mesi: età per i lavori usuranti (dipendenti).</t>
+        </is>
+      </c>
+      <c r="D57" s="27" t="inlineStr">
+        <is>
+          <t>fisso</t>
+        </is>
+      </c>
+      <c r="E57" s="27" t="inlineStr">
+        <is>
+          <t>eta&gt;=usurantiEta</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E57"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Excel: colonna Fonte (INPS / da richiedere all'interessato) nel foglio variabili
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZ53mE9kv9UaGeExs67Ewt
</commit_message>
<xml_diff>
--- a/motore/dati/Requisiti_domande_pensione.xlsx
+++ b/motore/dati/Requisiti_domande_pensione.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Variabili e fonti'!$A$4:$I$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Regole motore'!$A$1:$L$69</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Regole motore - variabili'!$A$1:$E$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Regole motore - variabili'!$A$1:$G$57</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <pivotCaches>
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,8 +81,11 @@
       <name val="Consolas"/>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -109,6 +112,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00003370"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F2FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F3F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="1" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -220,6 +238,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -16968,7 +16995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -17041,6 +17068,13 @@
       <c r="A10" t="inlineStr">
         <is>
           <t>Il significato di ogni variabile (condizioni, tipi di requisito, soglie) è nel foglio "Regole motore - variabili".</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Colonna "Fonte" del foglio variabili: INPS = dato presente negli archivi INPS (UNEX, ARCA, FELPE...); Da richiedere all'interessato = dato non disponibile negli archivi, da chiedere o dichiarare; Calcolata = derivata da altri dati; Normativa = parametro di legge.</t>
         </is>
       </c>
     </row>
@@ -17055,7 +17089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -17063,6 +17097,8 @@
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17091,6 +17127,16 @@
           <t>Esempio</t>
         </is>
       </c>
+      <c r="F1" s="25" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+      <c r="G1" s="25" t="inlineStr">
+        <is>
+          <t>Dettaglio della fonte</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="27" t="inlineStr">
@@ -17118,6 +17164,16 @@
           <t>Si applica se: ante96</t>
         </is>
       </c>
+      <c r="F2" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G2" s="27" t="inlineStr">
+        <is>
+          <t>UNEX / ARCA: anno del primo contributo</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="27" t="inlineStr">
@@ -17145,6 +17201,16 @@
           <t>Esclusa se: post95 =&gt; Primo contributo dopo il 1995.</t>
         </is>
       </c>
+      <c r="F3" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G3" s="27" t="inlineStr">
+        <is>
+          <t>UNEX / ARCA: anno del primo contributo</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
@@ -17172,6 +17238,16 @@
           <t>Si applica se: sesso.F</t>
         </is>
       </c>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>Anagrafica / codice fiscale</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -17199,6 +17275,16 @@
           <t>Si applica se: pensionato</t>
         </is>
       </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>Archivio pensioni: pensione diretta in essere</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
@@ -17226,6 +17312,16 @@
           <t>Si applica se: titolareAOI</t>
         </is>
       </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>Archivio pensioni: assegno ordinario di invalidità in essere</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
@@ -17253,6 +17349,16 @@
           <t>Si applica se: titolareInvalidita</t>
         </is>
       </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G7" s="27" t="inlineStr">
+        <is>
+          <t>Archivio pensioni: pensione di invalidità in essere</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
@@ -17280,6 +17386,16 @@
           <t>Si applica se: invalidita80</t>
         </is>
       </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G8" s="27" t="inlineStr">
+        <is>
+          <t>Archivio prestazioni/accertamenti medico-legali INPS, se già riconosciuta; altrimenti dichiarazione dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
@@ -17307,6 +17423,16 @@
           <t>Si applica se: editoria</t>
         </is>
       </c>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione: appartenenza al settore editoria e crisi aziendale</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
@@ -17334,6 +17460,16 @@
           <t>Si applica se: cert.VITTIMA_TERRORISMO; vittima80</t>
         </is>
       </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione: invalidità ≥ 80% riconosciuta dalla Prefettura (la certificazione di vittima è in FELPE)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
@@ -17361,6 +17497,16 @@
           <t>Si applica se: cert.VITTIMA_TERRORISMO; noVittima80</t>
         </is>
       </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione: invalidità &lt; 80% o familiare di vittima</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
@@ -17388,6 +17534,16 @@
           <t>Si applica se: ante96; noVecchiaiaOrdinaria</t>
         </is>
       </c>
+      <c r="F12" s="31" t="inlineStr">
+        <is>
+          <t>Calcolata</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>Calcolata da età e contributi (dati INPS)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
@@ -17415,6 +17571,16 @@
           <t>Si applica se: gest.AGO</t>
         </is>
       </c>
+      <c r="F13" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>UNEX: gestioni in cui ha versato</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
@@ -17442,6 +17608,16 @@
           <t>Si applica se: noGest.GS</t>
         </is>
       </c>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>UNEX: gestioni in cui ha versato</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
@@ -17469,6 +17645,16 @@
           <t>Si applica se: gest.ESCLUSIVA</t>
         </is>
       </c>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>UNEX / ex INPDAP: gestioni in cui ha versato</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
@@ -17496,6 +17682,16 @@
           <t>Si applica se: gest.CASSA</t>
         </is>
       </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>Le casse professionali private non sono negli archivi INPS: lo dichiara l'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
@@ -17523,6 +17719,16 @@
           <t>Si applica se: gest.ESTERO</t>
         </is>
       </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>La contribuzione estera non è negli archivi INPS: lo dichiara l'interessato (documentazione a suo carico)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
@@ -17550,6 +17756,16 @@
           <t>Si applica se: gsPiuAltre</t>
         </is>
       </c>
+      <c r="F18" s="31" t="inlineStr">
+        <is>
+          <t>Calcolata</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>Derivata dalle gestioni (INPS per AGO, GS ed esclusiva; dichiarata se coinvolge una cassa)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
@@ -17577,6 +17793,16 @@
           <t>Si applica se: cert.PRECOCI</t>
         </is>
       </c>
+      <c r="F19" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>FELPE: certificazione</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
@@ -17604,6 +17830,16 @@
           <t>Si applica se: cert.USURANTI</t>
         </is>
       </c>
+      <c r="F20" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>FELPE: certificazione</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
@@ -17631,6 +17867,16 @@
           <t>Si applica se: cert.GRAVOSI</t>
         </is>
       </c>
+      <c r="F21" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>FELPE: certificazione</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
@@ -17658,6 +17904,16 @@
           <t>Si applica se: cert.AMIANTO</t>
         </is>
       </c>
+      <c r="F22" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>FELPE: certificazione</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
@@ -17685,6 +17941,16 @@
           <t>Si applica se: ante96; cert.OPZIONE_CONTRIBUTIVO</t>
         </is>
       </c>
+      <c r="F23" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>FELPE: certificazione dell'opzione</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
@@ -17712,6 +17978,16 @@
           <t>Si applica se: cert.VITTIMA_TERRORISMO</t>
         </is>
       </c>
+      <c r="F24" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>FELPE: certificazione</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
@@ -17739,6 +18015,16 @@
           <t>Si applica se: cert.SALVAGUARDIA</t>
         </is>
       </c>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G25" s="27" t="inlineStr">
+        <is>
+          <t>FELPE: certificazione</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
@@ -17766,6 +18052,16 @@
           <t>Si applica se: salv.L214</t>
         </is>
       </c>
+      <c r="F26" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G26" s="27" t="inlineStr">
+        <is>
+          <t>FELPE: legge di salvaguardia certificata</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
@@ -17793,6 +18089,16 @@
           <t>Si applica se: deroga.contr92</t>
         </is>
       </c>
+      <c r="F27" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G27" s="27" t="inlineStr">
+        <is>
+          <t>UNEX: contributi maturati entro il 31/12/1992 (archivi storici; se mancano, si chiede all'interessato)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
@@ -17820,6 +18126,16 @@
           <t>una_tra(deroga.volontari92 : … ; …)</t>
         </is>
       </c>
+      <c r="F28" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G28" s="27" t="inlineStr">
+        <is>
+          <t>Archivio autorizzazioni ai versamenti volontari (archivi storici; se manca, si chiede all'interessato)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
@@ -17847,6 +18163,16 @@
           <t>una_tra(deroga.anz92 : … ; …)</t>
         </is>
       </c>
+      <c r="F29" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G29" s="27" t="inlineStr">
+        <is>
+          <t>UNEX: anzianità assicurativa al 1992 e primo contributo ante 1993 (archivi storici)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
@@ -17874,6 +18200,16 @@
           <t>Si applica se: deroga.qualsiasi</t>
         </is>
       </c>
+      <c r="F30" s="31" t="inlineStr">
+        <is>
+          <t>Calcolata</t>
+        </is>
+      </c>
+      <c r="G30" s="27" t="inlineStr">
+        <is>
+          <t>Derivata dalle tre condizioni sopra</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
@@ -17901,6 +18237,16 @@
           <t>Si applica se: grado.assoluta</t>
         </is>
       </c>
+      <c r="F31" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G31" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione dell'interessato; l'accertamento è dell'INPS in istruttoria</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
@@ -17928,6 +18274,16 @@
           <t>Esclusa se: causaServizio =&gt; …</t>
         </is>
       </c>
+      <c r="F32" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G32" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
@@ -17955,6 +18311,16 @@
           <t>Si applica se: marittimo</t>
         </is>
       </c>
+      <c r="F33" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G33" s="27" t="inlineStr">
+        <is>
+          <t>Gestione marittimi (ex IPSEMA) negli archivi INPS</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
@@ -17982,6 +18348,16 @@
           <t>Si applica se: soloRiconoscimento</t>
         </is>
       </c>
+      <c r="F34" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G34" s="27" t="inlineStr">
+        <is>
+          <t>Scelta dell'interessato: chiede solo il riconoscimento</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
@@ -18009,6 +18385,16 @@
           <t>Si applica se: dante.noPensionato</t>
         </is>
       </c>
+      <c r="F35" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G35" s="27" t="inlineStr">
+        <is>
+          <t>Archivio pensioni, una volta identificata la persona deceduta (il codice fiscale e il legame di parentela li indica l'interessato)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
@@ -18036,6 +18422,16 @@
           <t>Si applica se: dante.pensionato; dante.supplementare</t>
         </is>
       </c>
+      <c r="F36" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G36" s="27" t="inlineStr">
+        <is>
+          <t>Archivio pensioni del deceduto</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
@@ -18063,6 +18459,16 @@
           <t>Si applica se: dante.causaServizio</t>
         </is>
       </c>
+      <c r="F37" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G37" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
@@ -18090,6 +18496,16 @@
           <t>Si applica se: noMarittimoScomparso</t>
         </is>
       </c>
+      <c r="F38" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G38" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
@@ -18117,6 +18533,16 @@
           <t>Si applica se: dante.inabile</t>
         </is>
       </c>
+      <c r="F39" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G39" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione dell'interessato (inabilità al decesso)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
@@ -18144,6 +18570,16 @@
           <t>Si applica se: dante.estero</t>
         </is>
       </c>
+      <c r="F40" s="30" t="inlineStr">
+        <is>
+          <t>Da richiedere all'interessato</t>
+        </is>
+      </c>
+      <c r="G40" s="27" t="inlineStr">
+        <is>
+          <t>Dichiarazione dell'interessato: la contribuzione estera non è negli archivi INPS</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
@@ -18171,6 +18607,16 @@
           <t>Si applica se: dante.esclusiva</t>
         </is>
       </c>
+      <c r="F41" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G41" s="27" t="inlineStr">
+        <is>
+          <t>UNEX / ex INPDAP: gestioni del deceduto</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
@@ -18198,6 +18644,16 @@
           <t>Si applica se: dante.gsPiuAltre</t>
         </is>
       </c>
+      <c r="F42" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G42" s="27" t="inlineStr">
+        <is>
+          <t>UNEX: gestioni del deceduto</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
@@ -18225,6 +18681,16 @@
           <t>eta&gt;=vecchiaia =&gt; Servono {min} di età (hai {x}).</t>
         </is>
       </c>
+      <c r="F43" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G43" s="27" t="inlineStr">
+        <is>
+          <t>Anagrafica / codice fiscale: data di nascita</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
@@ -18252,6 +18718,16 @@
           <t>contr&gt;=20a =&gt; Servono 20 anni di contributi.</t>
         </is>
       </c>
+      <c r="F44" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
+        </is>
+      </c>
+      <c r="G44" s="27" t="inlineStr">
+        <is>
+          <t>UNEX: anzianità contributiva</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
@@ -18279,6 +18755,16 @@
           <t>quota&gt;=97.6 =&gt; Quota {min} (hai {x}).</t>
         </is>
       </c>
+      <c r="F45" s="31" t="inlineStr">
+        <is>
+          <t>Calcolata</t>
+        </is>
+      </c>
+      <c r="G45" s="27" t="inlineStr">
+        <is>
+          <t>Calcolata da età e contributi</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
@@ -18306,6 +18792,16 @@
           <t>contr@31/12/2025&gt;=41a =&gt; …</t>
         </is>
       </c>
+      <c r="F46" s="31" t="inlineStr">
+        <is>
+          <t>Calcolata</t>
+        </is>
+      </c>
+      <c r="G46" s="27" t="inlineStr">
+        <is>
+          <t>Calcolata da età e contributi (stima assumendo contribuzione continua)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
@@ -18333,6 +18829,16 @@
           <t>una_tra(deroga.contr92 : 15 anni al 1992 ; deroga.anz92 : 25 anni di anzianità) =&gt; Serve una tra…</t>
         </is>
       </c>
+      <c r="F47" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G47" s="27" t="inlineStr">
+        <is>
+          <t>Costrutto di scrittura delle regole: non è un dato</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
@@ -18360,6 +18866,16 @@
           <t>contr&gt;=20a</t>
         </is>
       </c>
+      <c r="F48" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G48" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
@@ -18387,6 +18903,16 @@
           <t>eta&gt;=M:61a/F:56a</t>
         </is>
       </c>
+      <c r="F49" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G49" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
@@ -18414,6 +18940,16 @@
           <t>quota&gt;=97.6</t>
         </is>
       </c>
+      <c r="F50" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G50" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
@@ -18441,6 +18977,16 @@
           <t>eta&gt;=vecchiaia</t>
         </is>
       </c>
+      <c r="F51" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G51" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
@@ -18468,6 +19014,16 @@
           <t>eta&gt;=vecchiaiaContributiva71</t>
         </is>
       </c>
+      <c r="F52" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G52" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
@@ -18495,6 +19051,16 @@
           <t>eta&gt;=contributiva64</t>
         </is>
       </c>
+      <c r="F53" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G53" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
@@ -18522,6 +19088,16 @@
           <t>contr&gt;=anticipata</t>
         </is>
       </c>
+      <c r="F54" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G54" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
@@ -18549,6 +19125,16 @@
           <t>contr&gt;=precoci</t>
         </is>
       </c>
+      <c r="F55" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G55" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
@@ -18576,6 +19162,16 @@
           <t>eta&gt;=gravosiEta</t>
         </is>
       </c>
+      <c r="F56" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G56" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
@@ -18603,9 +19199,19 @@
           <t>eta&gt;=usurantiEta</t>
         </is>
       </c>
+      <c r="F57" s="31" t="inlineStr">
+        <is>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G57" s="27" t="inlineStr">
+        <is>
+          <t>Parametro di legge: non è un dato dell'interessato</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E57"/>
+  <autoFilter ref="A1:G57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Excel: soglie e operatori con la fonte del dato verificato (INPS), niente più 'Normativa'
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZ53mE9kv9UaGeExs67Ewt
</commit_message>
<xml_diff>
--- a/motore/dati/Requisiti_domande_pensione.xlsx
+++ b/motore/dati/Requisiti_domande_pensione.xlsx
@@ -17074,7 +17074,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Colonna "Fonte" del foglio variabili: INPS = dato presente negli archivi INPS (UNEX, ARCA, FELPE...); Da richiedere all'interessato = dato non disponibile negli archivi, da chiedere o dichiarare; Calcolata = derivata da altri dati; Normativa = parametro di legge.</t>
+          <t>Colonna "Fonte" del foglio variabili: INPS = il dato che serve a verificare la condizione è negli archivi INPS (UNEX per i contributi, codice fiscale/anagrafica per età e sesso, FELPE per le certificazioni, archivio pensioni); Da richiedere all'interessato = il dato non è negli archivi e va chiesto o dichiarato. Soglie, parametri di legge e operatori (OR, quota) non sono dati: la fonte indicata è quella del dato su cui si verificano.</t>
         </is>
       </c>
     </row>
@@ -17534,14 +17534,14 @@
           <t>Si applica se: ante96; noVecchiaiaOrdinaria</t>
         </is>
       </c>
-      <c r="F12" s="31" t="inlineStr">
-        <is>
-          <t>Calcolata</t>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G12" s="27" t="inlineStr">
         <is>
-          <t>Calcolata da età e contributi (dati INPS)</t>
+          <t>INPS: calcolata da età (codice fiscale) e contributi (UNEX)</t>
         </is>
       </c>
     </row>
@@ -17756,14 +17756,14 @@
           <t>Si applica se: gsPiuAltre</t>
         </is>
       </c>
-      <c r="F18" s="31" t="inlineStr">
-        <is>
-          <t>Calcolata</t>
+      <c r="F18" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G18" s="27" t="inlineStr">
         <is>
-          <t>Derivata dalle gestioni (INPS per AGO, GS ed esclusiva; dichiarata se coinvolge una cassa)</t>
+          <t>INPS per AGO, Gestione separata ed esclusiva (UNEX); se coinvolge una cassa privata la cassa va dichiarata dall'interessato</t>
         </is>
       </c>
     </row>
@@ -18200,14 +18200,14 @@
           <t>Si applica se: deroga.qualsiasi</t>
         </is>
       </c>
-      <c r="F30" s="31" t="inlineStr">
-        <is>
-          <t>Calcolata</t>
+      <c r="F30" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G30" s="27" t="inlineStr">
         <is>
-          <t>Derivata dalle tre condizioni sopra</t>
+          <t>INPS: derivata dalle tre condizioni Amato (UNEX e archivio autorizzazioni)</t>
         </is>
       </c>
     </row>
@@ -18755,14 +18755,14 @@
           <t>quota&gt;=97.6 =&gt; Quota {min} (hai {x}).</t>
         </is>
       </c>
-      <c r="F45" s="31" t="inlineStr">
-        <is>
-          <t>Calcolata</t>
+      <c r="F45" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G45" s="27" t="inlineStr">
         <is>
-          <t>Calcolata da età e contributi</t>
+          <t>INPS: calcolata da età (codice fiscale) e contributi (UNEX)</t>
         </is>
       </c>
     </row>
@@ -18792,21 +18792,21 @@
           <t>contr@31/12/2025&gt;=41a =&gt; …</t>
         </is>
       </c>
-      <c r="F46" s="31" t="inlineStr">
-        <is>
-          <t>Calcolata</t>
+      <c r="F46" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G46" s="27" t="inlineStr">
         <is>
-          <t>Calcolata da età e contributi (stima assumendo contribuzione continua)</t>
+          <t>INPS: età (codice fiscale) e contributi (UNEX) stimati alla data indicata, assumendo contribuzione continua</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>Tipo di requisito</t>
+          <t>Soglia / operatore</t>
         </is>
       </c>
       <c r="B47" s="28" t="inlineStr">
@@ -18816,34 +18816,30 @@
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>Il requisito è soddisfatto se almeno una delle condizioni elencate è vera.</t>
-        </is>
-      </c>
-      <c r="D47" s="27" t="inlineStr">
-        <is>
-          <t>condizioni sopra</t>
-        </is>
-      </c>
+          <t>Combina in OR due o più condizioni (basta che una sia vera). Il dato verificato è quello delle singole condizioni: nella deroga Amato sono contributi e autorizzazioni ai versamenti volontari al 1992.</t>
+        </is>
+      </c>
+      <c r="D47" s="27" t="n"/>
       <c r="E47" s="27" t="inlineStr">
         <is>
           <t>una_tra(deroga.contr92 : 15 anni al 1992 ; deroga.anz92 : 25 anni di anzianità) =&gt; Serve una tra…</t>
         </is>
       </c>
-      <c r="F47" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F47" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G47" s="27" t="inlineStr">
         <is>
-          <t>Costrutto di scrittura delle regole: non è un dato</t>
+          <t>INPS: UNEX e archivio autorizzazioni (le fonti delle singole condizioni)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>Soglia</t>
+          <t>Soglia su contributi</t>
         </is>
       </c>
       <c r="B48" s="28" t="inlineStr">
@@ -18853,7 +18849,7 @@
       </c>
       <c r="C48" s="27" t="inlineStr">
         <is>
-          <t>Soglia fissa in anni (a) o in mesi (m).</t>
+          <t>Verifica che i contributi (anzianità contributiva) raggiungano la soglia indicata in anni (a) o mesi (m).</t>
         </is>
       </c>
       <c r="D48" s="27" t="inlineStr">
@@ -18866,21 +18862,21 @@
           <t>contr&gt;=20a</t>
         </is>
       </c>
-      <c r="F48" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F48" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G48" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: UNEX, anzianità contributiva</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>Soglia</t>
+          <t>Soglia su età, per sesso</t>
         </is>
       </c>
       <c r="B49" s="28" t="inlineStr">
@@ -18890,7 +18886,7 @@
       </c>
       <c r="C49" s="27" t="inlineStr">
         <is>
-          <t>Soglia diversa per uomini (M) e donne (F).</t>
+          <t>Verifica che l'età raggiunga la soglia prevista per uomini (M) o donne (F).</t>
         </is>
       </c>
       <c r="D49" s="27" t="inlineStr">
@@ -18903,21 +18899,21 @@
           <t>eta&gt;=M:61a/F:56a</t>
         </is>
       </c>
-      <c r="F49" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F49" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G49" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: codice fiscale / anagrafica (data di nascita e sesso)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>Soglia</t>
+          <t>Soglia sulla quota</t>
         </is>
       </c>
       <c r="B50" s="28" t="inlineStr">
@@ -18927,7 +18923,7 @@
       </c>
       <c r="C50" s="27" t="inlineStr">
         <is>
-          <t>Numero puro: usato per la quota.</t>
+          <t>Verifica che la quota (età più contributi, in anni) raggiunga il valore indicato.</t>
         </is>
       </c>
       <c r="D50" s="27" t="inlineStr">
@@ -18940,21 +18936,21 @@
           <t>quota&gt;=97.6</t>
         </is>
       </c>
-      <c r="F50" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F50" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G50" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: UNEX per i contributi e codice fiscale per l'età</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>Soglia (parametro normativo)</t>
+          <t>Soglia sull'età</t>
         </is>
       </c>
       <c r="B51" s="28" t="inlineStr">
@@ -18964,7 +18960,7 @@
       </c>
       <c r="C51" s="27" t="inlineStr">
         <is>
-          <t>67 anni più l'adeguamento alla speranza di vita (+1 mese dal 2027, +3 dal 2028).</t>
+          <t>Età di vecchiaia: 67 anni più l'adeguamento alla speranza di vita (+1 mese dal 2027, +3 dal 2028).</t>
         </is>
       </c>
       <c r="D51" s="27" t="inlineStr">
@@ -18977,21 +18973,21 @@
           <t>eta&gt;=vecchiaia</t>
         </is>
       </c>
-      <c r="F51" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F51" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G51" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: codice fiscale / anagrafica (data di nascita)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>Soglia (parametro normativo)</t>
+          <t>Soglia sull'età</t>
         </is>
       </c>
       <c r="B52" s="28" t="inlineStr">
@@ -19014,21 +19010,21 @@
           <t>eta&gt;=vecchiaiaContributiva71</t>
         </is>
       </c>
-      <c r="F52" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F52" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G52" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: codice fiscale / anagrafica (data di nascita)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>Soglia (parametro normativo)</t>
+          <t>Soglia sull'età</t>
         </is>
       </c>
       <c r="B53" s="28" t="inlineStr">
@@ -19038,7 +19034,7 @@
       </c>
       <c r="C53" s="27" t="inlineStr">
         <is>
-          <t>64 anni più adeguamento: anticipata nel sistema contributivo puro (con 20 anni).</t>
+          <t>64 anni più adeguamento: anticipata nel sistema contributivo puro (con 20 anni di contributi).</t>
         </is>
       </c>
       <c r="D53" s="27" t="inlineStr">
@@ -19051,21 +19047,21 @@
           <t>eta&gt;=contributiva64</t>
         </is>
       </c>
-      <c r="F53" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F53" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G53" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: codice fiscale / anagrafica (data di nascita)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>Soglia (parametro normativo)</t>
+          <t>Soglia sui contributi, per sesso</t>
         </is>
       </c>
       <c r="B54" s="28" t="inlineStr">
@@ -19088,21 +19084,21 @@
           <t>contr&gt;=anticipata</t>
         </is>
       </c>
-      <c r="F54" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F54" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G54" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: UNEX per i contributi, codice fiscale per il sesso</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>Soglia (parametro normativo)</t>
+          <t>Soglia sui contributi</t>
         </is>
       </c>
       <c r="B55" s="28" t="inlineStr">
@@ -19125,21 +19121,21 @@
           <t>contr&gt;=precoci</t>
         </is>
       </c>
-      <c r="F55" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F55" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G55" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: UNEX, anzianità contributiva</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>Soglia (parametro normativo)</t>
+          <t>Soglia sull'età</t>
         </is>
       </c>
       <c r="B56" s="28" t="inlineStr">
@@ -19162,21 +19158,21 @@
           <t>eta&gt;=gravosiEta</t>
         </is>
       </c>
-      <c r="F56" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F56" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G56" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: codice fiscale / anagrafica (data di nascita)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>Soglia (parametro normativo)</t>
+          <t>Soglia sull'età</t>
         </is>
       </c>
       <c r="B57" s="28" t="inlineStr">
@@ -19199,14 +19195,14 @@
           <t>eta&gt;=usurantiEta</t>
         </is>
       </c>
-      <c r="F57" s="31" t="inlineStr">
-        <is>
-          <t>Normativa</t>
+      <c r="F57" s="29" t="inlineStr">
+        <is>
+          <t>INPS</t>
         </is>
       </c>
       <c r="G57" s="27" t="inlineStr">
         <is>
-          <t>Parametro di legge: non è un dato dell'interessato</t>
+          <t>INPS: codice fiscale / anagrafica (data di nascita)</t>
         </is>
       </c>
     </row>

</xml_diff>